<commit_message>
fix length calculate jps only euclidean
</commit_message>
<xml_diff>
--- a/Excel/Validasi/Hasil_Pengujian_Map_1_128_avg_length.xlsx
+++ b/Excel/Validasi/Hasil_Pengujian_Map_1_128_avg_length.xlsx
@@ -506,19 +506,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.0004756999999999999</v>
+        <v>0.000488</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0028988</v>
+        <v>0.002934</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0186209</v>
+        <v>0.0191111</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1221172</v>
+        <v>0.1264418</v>
       </c>
       <c r="G2" t="n">
-        <v>0.03602815</v>
+        <v>0.037243725</v>
       </c>
     </row>
     <row r="3">
@@ -531,19 +531,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.0003067</v>
+        <v>0.0003022</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0012662</v>
+        <v>0.0011951</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0048661</v>
+        <v>0.0049929</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0206463</v>
+        <v>0.0208262</v>
       </c>
       <c r="G3" t="n">
-        <v>0.006771325000000001</v>
+        <v>0.006829100000000001</v>
       </c>
     </row>
     <row r="4">
@@ -556,19 +556,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.0004619</v>
+        <v>0.0004053</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0020094</v>
+        <v>0.0018053</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0158992</v>
+        <v>0.0142213</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1740273</v>
+        <v>0.1646243</v>
       </c>
       <c r="G4" t="n">
-        <v>0.04809945</v>
+        <v>0.04526405</v>
       </c>
     </row>
     <row r="5">
@@ -581,19 +581,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.0003941</v>
+        <v>0.0003970999999999999</v>
       </c>
       <c r="D5" t="n">
-        <v>0.002353</v>
+        <v>0.0023637</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0155628</v>
+        <v>0.0155513</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1056073</v>
+        <v>0.1113312</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0309793</v>
+        <v>0.032410825</v>
       </c>
     </row>
     <row r="6">
@@ -606,19 +606,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.0003715</v>
+        <v>0.0003778</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0010265</v>
+        <v>0.0009717</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0033432</v>
+        <v>0.0033759</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0119062</v>
+        <v>0.012292</v>
       </c>
       <c r="G6" t="n">
-        <v>0.00416185</v>
+        <v>0.00425435</v>
       </c>
     </row>
     <row r="7">
@@ -631,19 +631,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.0005382000000000001</v>
+        <v>0.0006016000000000001</v>
       </c>
       <c r="D7" t="n">
-        <v>0.002879800000000001</v>
+        <v>0.003082</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0186637</v>
+        <v>0.0195018</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1220557</v>
+        <v>0.127873</v>
       </c>
       <c r="G7" t="n">
-        <v>0.03603435</v>
+        <v>0.0377646</v>
       </c>
     </row>
     <row r="8">
@@ -656,19 +656,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.0005308</v>
+        <v>0.0005254999999999999</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0028147</v>
+        <v>0.0027902</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0176039</v>
+        <v>0.0178527</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1156211</v>
+        <v>0.1198106</v>
       </c>
       <c r="G8" t="n">
-        <v>0.034142625</v>
+        <v>0.03524475</v>
       </c>
     </row>
     <row r="9">
@@ -681,19 +681,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.0004712</v>
+        <v>0.0004429</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0018196</v>
+        <v>0.0016992</v>
       </c>
       <c r="E9" t="n">
-        <v>0.008529600000000002</v>
+        <v>0.008820700000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>0.051552</v>
+        <v>0.0528004</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0155931</v>
+        <v>0.0159408</v>
       </c>
     </row>
     <row r="10">
@@ -706,19 +706,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.0003732</v>
+        <v>0.0003189</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0014352</v>
+        <v>0.0013871</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0058292</v>
+        <v>0.005935</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0246614</v>
+        <v>0.0249958</v>
       </c>
       <c r="G10" t="n">
-        <v>0.00807475</v>
+        <v>0.0081592</v>
       </c>
     </row>
     <row r="11">
@@ -731,19 +731,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.000318</v>
+        <v>0.0003365</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0013445</v>
+        <v>0.0013536</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0061563</v>
+        <v>0.005054500000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0210556</v>
+        <v>0.0217027</v>
       </c>
       <c r="G11" t="n">
-        <v>0.007218599999999999</v>
+        <v>0.007111825</v>
       </c>
     </row>
     <row r="12">
@@ -756,19 +756,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.0003443</v>
+        <v>0.0003193</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0015302</v>
+        <v>0.0014867</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0055171</v>
+        <v>0.0054447</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0218654</v>
+        <v>0.021916</v>
       </c>
       <c r="G12" t="n">
-        <v>0.00731425</v>
+        <v>0.007291674999999999</v>
       </c>
     </row>
     <row r="13">
@@ -781,19 +781,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.0004921</v>
+        <v>0.0004682000000000001</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0021853</v>
+        <v>0.0019299</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0167967</v>
+        <v>0.0142374</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1759747</v>
+        <v>0.1669026</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0488622</v>
+        <v>0.045884525</v>
       </c>
     </row>
     <row r="14">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.0005229</v>
+        <v>0.0004872</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0021296</v>
+        <v>0.001915</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0162308</v>
+        <v>0.0138306</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1649628</v>
+        <v>0.1616847</v>
       </c>
       <c r="G14" t="n">
-        <v>0.04596152499999999</v>
+        <v>0.04447937499999999</v>
       </c>
     </row>
     <row r="15">
@@ -831,19 +831,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.0005288</v>
+        <v>0.0005844</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0027433</v>
+        <v>0.0026095</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0204157</v>
+        <v>0.0183228</v>
       </c>
       <c r="F15" t="n">
-        <v>0.2079127</v>
+        <v>0.1764387</v>
       </c>
       <c r="G15" t="n">
-        <v>0.057900125</v>
+        <v>0.04948885</v>
       </c>
     </row>
     <row r="16">
@@ -856,19 +856,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.0004431</v>
+        <v>0.0004614</v>
       </c>
       <c r="D16" t="n">
-        <v>0.00235</v>
+        <v>0.00241</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0158109</v>
+        <v>0.0156817</v>
       </c>
       <c r="F16" t="n">
-        <v>0.106677</v>
+        <v>0.1132413</v>
       </c>
       <c r="G16" t="n">
-        <v>0.03132025</v>
+        <v>0.0329486</v>
       </c>
     </row>
     <row r="17">
@@ -881,19 +881,19 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.0005802</v>
+        <v>0.0005739</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0034873</v>
+        <v>0.0035986</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0157301</v>
+        <v>0.0158411</v>
       </c>
       <c r="F17" t="n">
-        <v>0.1034032</v>
+        <v>0.1056952</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0308002</v>
+        <v>0.0314272</v>
       </c>
     </row>
     <row r="18">
@@ -906,19 +906,19 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.0003467</v>
+        <v>0.0003591</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0009754000000000001</v>
+        <v>0.00098</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0028549</v>
+        <v>0.0028888</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0108609</v>
+        <v>0.0108466</v>
       </c>
       <c r="G18" t="n">
-        <v>0.003759475</v>
+        <v>0.003768625</v>
       </c>
     </row>
     <row r="19">
@@ -931,19 +931,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.0003091</v>
+        <v>0.0003145</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0008983</v>
+        <v>0.0008716999999999999</v>
       </c>
       <c r="E19" t="n">
-        <v>0.0032276</v>
+        <v>0.0025937</v>
       </c>
       <c r="F19" t="n">
-        <v>0.0117835</v>
+        <v>0.0121766</v>
       </c>
       <c r="G19" t="n">
-        <v>0.004054625</v>
+        <v>0.003989125</v>
       </c>
     </row>
     <row r="20">
@@ -956,19 +956,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.0003916999999999999</v>
+        <v>0.000361</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0011461</v>
+        <v>0.0011302</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0036688</v>
+        <v>0.0036276</v>
       </c>
       <c r="F20" t="n">
-        <v>0.0132597</v>
+        <v>0.0133442</v>
       </c>
       <c r="G20" t="n">
-        <v>0.004616574999999999</v>
+        <v>0.00461575</v>
       </c>
     </row>
     <row r="21">
@@ -981,19 +981,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.0003956</v>
+        <v>0.0003751</v>
       </c>
       <c r="D21" t="n">
-        <v>0.0010646</v>
+        <v>0.0011003</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0033574</v>
+        <v>0.0034493</v>
       </c>
       <c r="F21" t="n">
-        <v>0.012179</v>
+        <v>0.0122192</v>
       </c>
       <c r="G21" t="n">
-        <v>0.00424915</v>
+        <v>0.004285975</v>
       </c>
     </row>
     <row r="22">
@@ -1006,19 +1006,19 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.0005819</v>
+        <v>0.0005897000000000001</v>
       </c>
       <c r="D22" t="n">
-        <v>0.0028</v>
+        <v>0.0029227</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0177781</v>
+        <v>0.0182536</v>
       </c>
       <c r="F22" t="n">
-        <v>0.1173793</v>
+        <v>0.1212913</v>
       </c>
       <c r="G22" t="n">
-        <v>0.034634825</v>
+        <v>0.035764325</v>
       </c>
     </row>
     <row r="23">
@@ -1031,19 +1031,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.000505</v>
+        <v>0.0005002</v>
       </c>
       <c r="D23" t="n">
-        <v>0.0019143</v>
+        <v>0.0017475</v>
       </c>
       <c r="E23" t="n">
-        <v>0.008947300000000002</v>
+        <v>0.008291099999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0540928</v>
+        <v>0.0530564</v>
       </c>
       <c r="G23" t="n">
-        <v>0.01636485</v>
+        <v>0.0158988</v>
       </c>
     </row>
     <row r="24">
@@ -1056,19 +1056,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.0004673</v>
+        <v>0.0005290999999999999</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0020009</v>
+        <v>0.0017723</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0093343</v>
+        <v>0.0085497</v>
       </c>
       <c r="F24" t="n">
-        <v>0.054073</v>
+        <v>0.0533539</v>
       </c>
       <c r="G24" t="n">
-        <v>0.016468875</v>
+        <v>0.01605125</v>
       </c>
     </row>
     <row r="25">
@@ -1081,19 +1081,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.0005209</v>
+        <v>0.0005549</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0028063</v>
+        <v>0.0023584</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0136905</v>
+        <v>0.012572</v>
       </c>
       <c r="F25" t="n">
-        <v>0.08627009999999999</v>
+        <v>0.0846522</v>
       </c>
       <c r="G25" t="n">
-        <v>0.02582195</v>
+        <v>0.025034375</v>
       </c>
     </row>
     <row r="26">
@@ -1106,19 +1106,19 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.0003688</v>
+        <v>0.0003788</v>
       </c>
       <c r="D26" t="n">
-        <v>0.0015198</v>
+        <v>0.0015154</v>
       </c>
       <c r="E26" t="n">
-        <v>0.006096</v>
+        <v>0.006075</v>
       </c>
       <c r="F26" t="n">
-        <v>0.0252678</v>
+        <v>0.0262154</v>
       </c>
       <c r="G26" t="n">
-        <v>0.0083131</v>
+        <v>0.008546149999999999</v>
       </c>
     </row>
     <row r="27">
@@ -1131,19 +1131,19 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.0003525</v>
+        <v>0.0003761</v>
       </c>
       <c r="D27" t="n">
-        <v>0.0016157</v>
+        <v>0.0016044</v>
       </c>
       <c r="E27" t="n">
-        <v>0.0065068</v>
+        <v>0.0063856</v>
       </c>
       <c r="F27" t="n">
-        <v>0.02576230000000001</v>
+        <v>0.0264375</v>
       </c>
       <c r="G27" t="n">
-        <v>0.008559325000000001</v>
+        <v>0.008700899999999999</v>
       </c>
     </row>
     <row r="28">
@@ -1156,19 +1156,19 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.0003619</v>
+        <v>0.000369</v>
       </c>
       <c r="D28" t="n">
-        <v>0.0015598</v>
+        <v>0.0015119</v>
       </c>
       <c r="E28" t="n">
-        <v>0.0057539</v>
+        <v>0.005735599999999999</v>
       </c>
       <c r="F28" t="n">
-        <v>0.0223897</v>
+        <v>0.0228551</v>
       </c>
       <c r="G28" t="n">
-        <v>0.007516324999999999</v>
+        <v>0.007617899999999999</v>
       </c>
     </row>
     <row r="29">
@@ -1181,19 +1181,19 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.0005151</v>
+        <v>0.0005112000000000001</v>
       </c>
       <c r="D29" t="n">
-        <v>0.0023147</v>
+        <v>0.0020943</v>
       </c>
       <c r="E29" t="n">
-        <v>0.0165782</v>
+        <v>0.0142882</v>
       </c>
       <c r="F29" t="n">
-        <v>0.1687278</v>
+        <v>0.1643884</v>
       </c>
       <c r="G29" t="n">
-        <v>0.04703395</v>
+        <v>0.045320525</v>
       </c>
     </row>
     <row r="30">
@@ -1206,19 +1206,19 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.0005317000000000001</v>
+        <v>0.0006200999999999999</v>
       </c>
       <c r="D30" t="n">
-        <v>0.0028494</v>
+        <v>0.0025644</v>
       </c>
       <c r="E30" t="n">
-        <v>0.0209271</v>
+        <v>0.0187376</v>
       </c>
       <c r="F30" t="n">
-        <v>0.2072366</v>
+        <v>0.179151</v>
       </c>
       <c r="G30" t="n">
-        <v>0.05788620000000001</v>
+        <v>0.050268275</v>
       </c>
     </row>
     <row r="31">
@@ -1231,19 +1231,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.0005666000000000001</v>
+        <v>0.0006041</v>
       </c>
       <c r="D31" t="n">
-        <v>0.0028583</v>
+        <v>0.0027139</v>
       </c>
       <c r="E31" t="n">
-        <v>0.0213642</v>
+        <v>0.0179335</v>
       </c>
       <c r="F31" t="n">
-        <v>0.2053403</v>
+        <v>0.1518734</v>
       </c>
       <c r="G31" t="n">
-        <v>0.05753235</v>
+        <v>0.043281225</v>
       </c>
     </row>
     <row r="32">
@@ -1256,19 +1256,19 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.0006046000000000001</v>
+        <v>0.0006119</v>
       </c>
       <c r="D32" t="n">
-        <v>0.0035056</v>
+        <v>0.0035223</v>
       </c>
       <c r="E32" t="n">
-        <v>0.0163175</v>
+        <v>0.0160673</v>
       </c>
       <c r="F32" t="n">
-        <v>0.1051713</v>
+        <v>0.1078077</v>
       </c>
       <c r="G32" t="n">
-        <v>0.03139975</v>
+        <v>0.0320023</v>
       </c>
     </row>
     <row r="33">
@@ -1281,19 +1281,19 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0.0004681</v>
+        <v>0.0004094</v>
       </c>
       <c r="D33" t="n">
-        <v>0.0011065</v>
+        <v>0.0011284</v>
       </c>
       <c r="E33" t="n">
-        <v>0.0033254</v>
+        <v>0.0032717</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0117152</v>
+        <v>0.0107584</v>
       </c>
       <c r="G33" t="n">
-        <v>0.004153799999999999</v>
+        <v>0.003891975</v>
       </c>
     </row>
     <row r="34">
@@ -1306,19 +1306,19 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0.0003272</v>
+        <v>0.0003128000000000001</v>
       </c>
       <c r="D34" t="n">
-        <v>0.0011511</v>
+        <v>0.0010323</v>
       </c>
       <c r="E34" t="n">
-        <v>0.0029128</v>
+        <v>0.0029806</v>
       </c>
       <c r="F34" t="n">
-        <v>0.0112634</v>
+        <v>0.0113632</v>
       </c>
       <c r="G34" t="n">
-        <v>0.003913625</v>
+        <v>0.003922225000000001</v>
       </c>
     </row>
     <row r="35">
@@ -1331,19 +1331,19 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.0003986000000000001</v>
+        <v>0.0004091</v>
       </c>
       <c r="D35" t="n">
-        <v>0.0010193</v>
+        <v>0.0009947999999999999</v>
       </c>
       <c r="E35" t="n">
-        <v>0.0030416</v>
+        <v>0.0029447</v>
       </c>
       <c r="F35" t="n">
-        <v>0.0108127</v>
+        <v>0.0111221</v>
       </c>
       <c r="G35" t="n">
-        <v>0.00381805</v>
+        <v>0.003867675</v>
       </c>
     </row>
     <row r="36">
@@ -1356,19 +1356,19 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0.0003326</v>
+        <v>0.0003565</v>
       </c>
       <c r="D36" t="n">
-        <v>0.0009556</v>
+        <v>0.0009288999999999999</v>
       </c>
       <c r="E36" t="n">
-        <v>0.0032688</v>
+        <v>0.0025786</v>
       </c>
       <c r="F36" t="n">
-        <v>0.0117226</v>
+        <v>0.0121538</v>
       </c>
       <c r="G36" t="n">
-        <v>0.0040699</v>
+        <v>0.00400445</v>
       </c>
     </row>
     <row r="37">
@@ -1381,19 +1381,19 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0.0003278</v>
+        <v>0.000322</v>
       </c>
       <c r="D37" t="n">
-        <v>0.0010643</v>
+        <v>0.0009711000000000001</v>
       </c>
       <c r="E37" t="n">
-        <v>0.002871</v>
+        <v>0.0026808</v>
       </c>
       <c r="F37" t="n">
-        <v>0.0125853</v>
+        <v>0.0114559</v>
       </c>
       <c r="G37" t="n">
-        <v>0.0042121</v>
+        <v>0.00385745</v>
       </c>
     </row>
     <row r="38">
@@ -1406,19 +1406,19 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0.0004063000000000001</v>
+        <v>0.0004107000000000001</v>
       </c>
       <c r="D38" t="n">
-        <v>0.0011827</v>
+        <v>0.0012051</v>
       </c>
       <c r="E38" t="n">
-        <v>0.0037134</v>
+        <v>0.0036779</v>
       </c>
       <c r="F38" t="n">
-        <v>0.0132234</v>
+        <v>0.0133779</v>
       </c>
       <c r="G38" t="n">
-        <v>0.00463145</v>
+        <v>0.004667900000000001</v>
       </c>
     </row>
     <row r="39">
@@ -1431,19 +1431,19 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0.0004917000000000001</v>
+        <v>0.0005093000000000001</v>
       </c>
       <c r="D39" t="n">
-        <v>0.0020552</v>
+        <v>0.0019482</v>
       </c>
       <c r="E39" t="n">
-        <v>0.0096069</v>
+        <v>0.0090095</v>
       </c>
       <c r="F39" t="n">
-        <v>0.0543331</v>
+        <v>0.05484220000000001</v>
       </c>
       <c r="G39" t="n">
-        <v>0.016621725</v>
+        <v>0.0165773</v>
       </c>
     </row>
     <row r="40">
@@ -1456,19 +1456,19 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0.0005229</v>
+        <v>0.0005922</v>
       </c>
       <c r="D40" t="n">
-        <v>0.00289</v>
+        <v>0.0023443</v>
       </c>
       <c r="E40" t="n">
-        <v>0.0140074</v>
+        <v>0.0129631</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0875451</v>
+        <v>0.0861218</v>
       </c>
       <c r="G40" t="n">
-        <v>0.02624135</v>
+        <v>0.02550535</v>
       </c>
     </row>
     <row r="41">
@@ -1481,19 +1481,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0.000592</v>
+        <v>0.0006981</v>
       </c>
       <c r="D41" t="n">
-        <v>0.003019399999999999</v>
+        <v>0.002830099999999999</v>
       </c>
       <c r="E41" t="n">
-        <v>0.0147816</v>
+        <v>0.0139667</v>
       </c>
       <c r="F41" t="n">
-        <v>0.0860274</v>
+        <v>0.085648</v>
       </c>
       <c r="G41" t="n">
-        <v>0.0261051</v>
+        <v>0.025785725</v>
       </c>
     </row>
     <row r="42">
@@ -1506,19 +1506,19 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.0004217</v>
+        <v>0.000403</v>
       </c>
       <c r="D42" t="n">
-        <v>0.0017371</v>
+        <v>0.001654</v>
       </c>
       <c r="E42" t="n">
-        <v>0.0066523</v>
+        <v>0.0066898</v>
       </c>
       <c r="F42" t="n">
-        <v>0.0264875</v>
+        <v>0.0271707</v>
       </c>
       <c r="G42" t="n">
-        <v>0.00882465</v>
+        <v>0.008979375</v>
       </c>
     </row>
     <row r="43">
@@ -1531,19 +1531,19 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0.0006101</v>
+        <v>0.0006057</v>
       </c>
       <c r="D43" t="n">
-        <v>0.002870699999999999</v>
+        <v>0.0028399</v>
       </c>
       <c r="E43" t="n">
-        <v>0.0220386</v>
+        <v>0.0179021</v>
       </c>
       <c r="F43" t="n">
-        <v>0.2044078</v>
+        <v>0.1528052</v>
       </c>
       <c r="G43" t="n">
-        <v>0.05748179999999999</v>
+        <v>0.04353822500000001</v>
       </c>
     </row>
     <row r="44">
@@ -1556,19 +1556,19 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0.0004442</v>
+        <v>0.0003966</v>
       </c>
       <c r="D44" t="n">
-        <v>0.0012349</v>
+        <v>0.0011272</v>
       </c>
       <c r="E44" t="n">
-        <v>0.0033418</v>
+        <v>0.0032949</v>
       </c>
       <c r="F44" t="n">
-        <v>0.0113932</v>
+        <v>0.0106684</v>
       </c>
       <c r="G44" t="n">
-        <v>0.004103525</v>
+        <v>0.003871775</v>
       </c>
     </row>
     <row r="45">
@@ -1581,19 +1581,19 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0.0003973</v>
+        <v>0.0004068</v>
       </c>
       <c r="D45" t="n">
-        <v>0.0014864</v>
+        <v>0.0014149</v>
       </c>
       <c r="E45" t="n">
-        <v>0.0036257</v>
+        <v>0.0033747</v>
       </c>
       <c r="F45" t="n">
-        <v>0.0128792</v>
+        <v>0.0117605</v>
       </c>
       <c r="G45" t="n">
-        <v>0.00459715</v>
+        <v>0.004239224999999999</v>
       </c>
     </row>
     <row r="46">
@@ -1606,19 +1606,19 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.0003356</v>
+        <v>0.0003226</v>
       </c>
       <c r="D46" t="n">
-        <v>0.0011823</v>
+        <v>0.0010937</v>
       </c>
       <c r="E46" t="n">
-        <v>0.0030179</v>
+        <v>0.0030327</v>
       </c>
       <c r="F46" t="n">
-        <v>0.0115555</v>
+        <v>0.0113453</v>
       </c>
       <c r="G46" t="n">
-        <v>0.004022825</v>
+        <v>0.003948574999999999</v>
       </c>
     </row>
     <row r="47">
@@ -1631,19 +1631,19 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0.0003649</v>
+        <v>0.0003851</v>
       </c>
       <c r="D47" t="n">
-        <v>0.0010953</v>
+        <v>0.0010217</v>
       </c>
       <c r="E47" t="n">
-        <v>0.00299</v>
+        <v>0.0027238</v>
       </c>
       <c r="F47" t="n">
-        <v>0.0123946</v>
+        <v>0.0114242</v>
       </c>
       <c r="G47" t="n">
-        <v>0.0042112</v>
+        <v>0.0038887</v>
       </c>
     </row>
     <row r="48">
@@ -1656,19 +1656,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.0006339000000000001</v>
+        <v>0.0007373</v>
       </c>
       <c r="D48" t="n">
-        <v>0.0032533</v>
+        <v>0.0029201</v>
       </c>
       <c r="E48" t="n">
-        <v>0.0148296</v>
+        <v>0.0142106</v>
       </c>
       <c r="F48" t="n">
-        <v>0.08674019999999998</v>
+        <v>0.0864718</v>
       </c>
       <c r="G48" t="n">
-        <v>0.02636425</v>
+        <v>0.02608495</v>
       </c>
     </row>
     <row r="49">
@@ -1681,19 +1681,19 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0.0004256</v>
+        <v>0.0004337</v>
       </c>
       <c r="D49" t="n">
-        <v>0.0014189</v>
+        <v>0.001344</v>
       </c>
       <c r="E49" t="n">
-        <v>0.0037633</v>
+        <v>0.003318</v>
       </c>
       <c r="F49" t="n">
-        <v>0.0128954</v>
+        <v>0.0118754</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0046258</v>
+        <v>0.004242775</v>
       </c>
     </row>
   </sheetData>
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4" t="n">
         <v>44</v>
@@ -1819,7 +1819,7 @@
         <v>176</v>
       </c>
       <c r="G4" t="n">
-        <v>82.75</v>
+        <v>82.5</v>
       </c>
     </row>
     <row r="5">
@@ -2032,7 +2032,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D13" t="n">
         <v>8</v>
@@ -2044,7 +2044,7 @@
         <v>9</v>
       </c>
       <c r="G13" t="n">
-        <v>8.75</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="14">
@@ -2082,10 +2082,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D15" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E15" t="n">
         <v>96</v>
@@ -2094,7 +2094,7 @@
         <v>192</v>
       </c>
       <c r="G15" t="n">
-        <v>88.5</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16">
@@ -2182,19 +2182,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D19" t="n">
         <v>20</v>
       </c>
       <c r="E19" t="n">
+        <v>20</v>
+      </c>
+      <c r="F19" t="n">
         <v>21</v>
       </c>
-      <c r="F19" t="n">
+      <c r="G19" t="n">
         <v>20</v>
-      </c>
-      <c r="G19" t="n">
-        <v>19.75</v>
       </c>
     </row>
     <row r="20">
@@ -2232,19 +2232,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D21" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F21" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G21" t="n">
-        <v>8.5</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="22">
@@ -2335,7 +2335,7 @@
         <v>24</v>
       </c>
       <c r="D25" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E25" t="n">
         <v>96</v>
@@ -2344,7 +2344,7 @@
         <v>192</v>
       </c>
       <c r="G25" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="26">
@@ -2457,10 +2457,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D30" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E30" t="n">
         <v>9</v>
@@ -2469,7 +2469,7 @@
         <v>9</v>
       </c>
       <c r="G30" t="n">
-        <v>9</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="31">
@@ -2488,13 +2488,13 @@
         <v>44</v>
       </c>
       <c r="E31" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="F31" t="n">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="G31" t="n">
-        <v>88.5</v>
+        <v>82.5</v>
       </c>
     </row>
     <row r="32">
@@ -2582,19 +2582,19 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D35" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E35" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F35" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G35" t="n">
-        <v>7.75</v>
+        <v>8.75</v>
       </c>
     </row>
     <row r="36">
@@ -2607,19 +2607,19 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D36" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E36" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F36" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G36" t="n">
-        <v>10.5</v>
+        <v>11.75</v>
       </c>
     </row>
     <row r="37">
@@ -2657,19 +2657,19 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D38" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F38" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G38" t="n">
-        <v>8.25</v>
+        <v>9.25</v>
       </c>
     </row>
     <row r="39">
@@ -2707,10 +2707,10 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D40" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E40" t="n">
         <v>10</v>
@@ -2719,7 +2719,7 @@
         <v>10</v>
       </c>
       <c r="G40" t="n">
-        <v>9.5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41">
@@ -2732,19 +2732,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D41" t="n">
         <v>44</v>
       </c>
       <c r="E41" t="n">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="F41" t="n">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="G41" t="n">
-        <v>89</v>
+        <v>82.5</v>
       </c>
     </row>
     <row r="42">
@@ -2782,19 +2782,19 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D43" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E43" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F43" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G43" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="44">
@@ -2807,19 +2807,19 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D44" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E44" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F44" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G44" t="n">
-        <v>8.75</v>
+        <v>10.25</v>
       </c>
     </row>
     <row r="45">
@@ -2857,19 +2857,19 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D46" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E46" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F46" t="n">
+        <v>11</v>
+      </c>
+      <c r="G46" t="n">
         <v>10</v>
-      </c>
-      <c r="G46" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="47">
@@ -2882,19 +2882,19 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D47" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E47" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F47" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G47" t="n">
-        <v>9.5</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="48">
@@ -2907,19 +2907,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D48" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E48" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F48" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G48" t="n">
-        <v>9.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="49">
@@ -2932,19 +2932,19 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D49" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E49" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F49" t="n">
+        <v>11</v>
+      </c>
+      <c r="G49" t="n">
         <v>10</v>
-      </c>
-      <c r="G49" t="n">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -3058,7 +3058,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>26.97056274847714</v>
+        <v>25.55634918610405</v>
       </c>
       <c r="D4" t="n">
         <v>52.52691193458119</v>
@@ -3070,7 +3070,7 @@
         <v>214.350288425444</v>
       </c>
       <c r="G4" t="n">
-        <v>100.0789501350095</v>
+        <v>99.72539674441619</v>
       </c>
     </row>
     <row r="5">
@@ -3186,7 +3186,7 @@
         <v>25.55634918610405</v>
       </c>
       <c r="D9" t="n">
-        <v>53.35533905932738</v>
+        <v>52.52691193458119</v>
       </c>
       <c r="E9" t="n">
         <v>107.2964645562817</v>
@@ -3195,7 +3195,7 @@
         <v>215.1787155501902</v>
       </c>
       <c r="G9" t="n">
-        <v>100.3467170879758</v>
+        <v>100.1396103067893</v>
       </c>
     </row>
     <row r="10">
@@ -3283,7 +3283,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>25.7850865361163</v>
+        <v>24.41488446708389</v>
       </c>
       <c r="D13" t="n">
         <v>49.56011556674471</v>
@@ -3295,7 +3295,7 @@
         <v>203.2348880049742</v>
       </c>
       <c r="G13" t="n">
-        <v>94.92412607931394</v>
+        <v>94.58157556205583</v>
       </c>
     </row>
     <row r="14">
@@ -3333,19 +3333,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>25.55634918610405</v>
+        <v>27.55634918610405</v>
       </c>
       <c r="D15" t="n">
-        <v>51.69848480983499</v>
+        <v>54.87005768508881</v>
       </c>
       <c r="E15" t="n">
-        <v>109.4974746830583</v>
+        <v>108.6690475583121</v>
       </c>
       <c r="F15" t="n">
-        <v>218.7523086789974</v>
+        <v>217.9238815542512</v>
       </c>
       <c r="G15" t="n">
-        <v>101.3761543394987</v>
+        <v>102.254833995939</v>
       </c>
     </row>
     <row r="16">
@@ -3433,19 +3433,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>26.97056274847714</v>
+        <v>27.55634918610405</v>
       </c>
       <c r="D19" t="n">
         <v>54.04163056034262</v>
       </c>
       <c r="E19" t="n">
-        <v>111.8406204335659</v>
+        <v>108.6690475583121</v>
       </c>
       <c r="F19" t="n">
-        <v>217.9238815542512</v>
+        <v>223.4386001800126</v>
       </c>
       <c r="G19" t="n">
-        <v>102.6941738241592</v>
+        <v>103.4264068711929</v>
       </c>
     </row>
     <row r="20">
@@ -3483,19 +3483,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>23.74064110506006</v>
+        <v>24.62280887594792</v>
       </c>
       <c r="D21" t="n">
-        <v>50.17676995799587</v>
+        <v>50.84539750584248</v>
       </c>
       <c r="E21" t="n">
-        <v>100.1430788450122</v>
+        <v>101.6414365392452</v>
       </c>
       <c r="F21" t="n">
-        <v>200.8525404962239</v>
+        <v>204.0006534257569</v>
       </c>
       <c r="G21" t="n">
-        <v>93.72825760107301</v>
+        <v>95.27757408669811</v>
       </c>
     </row>
     <row r="22">
@@ -3536,7 +3536,7 @@
         <v>24.41488446708389</v>
       </c>
       <c r="D23" t="n">
-        <v>49.78173998791892</v>
+        <v>49.60484583115361</v>
       </c>
       <c r="E23" t="n">
         <v>101.1765739559945</v>
@@ -3545,7 +3545,7 @@
         <v>203.3015774098458</v>
       </c>
       <c r="G23" t="n">
-        <v>94.66869395521077</v>
+        <v>94.62447041601945</v>
       </c>
     </row>
     <row r="24">
@@ -3586,16 +3586,16 @@
         <v>27.55634918610405</v>
       </c>
       <c r="D25" t="n">
-        <v>52.52691193458119</v>
+        <v>54.04163056034262</v>
       </c>
       <c r="E25" t="n">
-        <v>110.3259018078045</v>
+        <v>109.4974746830583</v>
       </c>
       <c r="F25" t="n">
-        <v>219.5807358037436</v>
+        <v>218.7523086789974</v>
       </c>
       <c r="G25" t="n">
-        <v>102.4974746830583</v>
+        <v>102.4619407771256</v>
       </c>
     </row>
     <row r="26">
@@ -3689,13 +3689,13 @@
         <v>49.56011556674471</v>
       </c>
       <c r="E29" t="n">
-        <v>101.1164142094206</v>
+        <v>100.6044505332257</v>
       </c>
       <c r="F29" t="n">
         <v>203.2348880049742</v>
       </c>
       <c r="G29" t="n">
-        <v>94.58157556205583</v>
+        <v>94.45358464300712</v>
       </c>
     </row>
     <row r="30">
@@ -3708,19 +3708,19 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>24.41811047550525</v>
+        <v>25.83232403787834</v>
       </c>
       <c r="D30" t="n">
-        <v>49.04921408900104</v>
+        <v>51.44598283082938</v>
       </c>
       <c r="E30" t="n">
-        <v>103.7222775834009</v>
+        <v>103.0023916359005</v>
       </c>
       <c r="F30" t="n">
-        <v>207.7440267546941</v>
+        <v>206.425148898921</v>
       </c>
       <c r="G30" t="n">
-        <v>96.23340722565031</v>
+        <v>96.6764618508823</v>
       </c>
     </row>
     <row r="31">
@@ -3739,13 +3739,13 @@
         <v>51.69848480983499</v>
       </c>
       <c r="E31" t="n">
-        <v>109.4974746830583</v>
+        <v>103.9827560572969</v>
       </c>
       <c r="F31" t="n">
-        <v>218.7523086789974</v>
+        <v>208.5512985522207</v>
       </c>
       <c r="G31" t="n">
-        <v>101.3761543394987</v>
+        <v>97.44722215136416</v>
       </c>
     </row>
     <row r="32">
@@ -3783,7 +3783,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>25.55634918610405</v>
+        <v>27.55634918610405</v>
       </c>
       <c r="D33" t="n">
         <v>54.04163056034262</v>
@@ -3795,7 +3795,7 @@
         <v>217.9238815542512</v>
       </c>
       <c r="G33" t="n">
-        <v>101.5477272147525</v>
+        <v>102.0477272147525</v>
       </c>
     </row>
     <row r="34">
@@ -3833,19 +3833,19 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>23.53271669619603</v>
+        <v>24.41488446708389</v>
       </c>
       <c r="D35" t="n">
-        <v>49.50528473946896</v>
+        <v>50.17391228731556</v>
       </c>
       <c r="E35" t="n">
-        <v>98.58961006939111</v>
+        <v>100.087967763624</v>
       </c>
       <c r="F35" t="n">
-        <v>197.5695114409684</v>
+        <v>200.7176243705014</v>
       </c>
       <c r="G35" t="n">
-        <v>92.29928073650612</v>
+        <v>93.84859722213122</v>
       </c>
     </row>
     <row r="36">
@@ -3858,19 +3858,19 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>24.90291876522843</v>
+        <v>26.59251907515131</v>
       </c>
       <c r="D36" t="n">
-        <v>51.95837796962023</v>
+        <v>52.62700551746683</v>
       </c>
       <c r="E36" t="n">
-        <v>109.6176879416777</v>
+        <v>105.9675221282317</v>
       </c>
       <c r="F36" t="n">
-        <v>209.6068123063317</v>
+        <v>222.6622168960765</v>
       </c>
       <c r="G36" t="n">
-        <v>99.02144924571451</v>
+        <v>101.9623159042316</v>
       </c>
     </row>
     <row r="37">
@@ -3908,19 +3908,19 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>24.50457312756027</v>
+        <v>25.38674089844813</v>
       </c>
       <c r="D38" t="n">
-        <v>50.17676995799587</v>
+        <v>50.84539750584248</v>
       </c>
       <c r="E38" t="n">
-        <v>100.1430788450122</v>
+        <v>101.6414365392452</v>
       </c>
       <c r="F38" t="n">
-        <v>200.8525404962239</v>
+        <v>204.0006534257569</v>
       </c>
       <c r="G38" t="n">
-        <v>93.91924060669805</v>
+        <v>95.46855709232315</v>
       </c>
     </row>
     <row r="39">
@@ -3939,13 +3939,13 @@
         <v>49.56011556674471</v>
       </c>
       <c r="E39" t="n">
-        <v>101.1318436915856</v>
+        <v>100.6198800153907</v>
       </c>
       <c r="F39" t="n">
         <v>203.2568471454369</v>
       </c>
       <c r="G39" t="n">
-        <v>94.59092271771277</v>
+        <v>94.46293179866406</v>
       </c>
     </row>
     <row r="40">
@@ -3958,19 +3958,19 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>26.07297705925549</v>
+        <v>25.71936168599622</v>
       </c>
       <c r="D40" t="n">
-        <v>49.24441272425872</v>
+        <v>51.44598283082938</v>
       </c>
       <c r="E40" t="n">
-        <v>103.8198470130748</v>
+        <v>103.0999610655744</v>
       </c>
       <c r="F40" t="n">
-        <v>207.8890363034826</v>
+        <v>206.5701584477096</v>
       </c>
       <c r="G40" t="n">
-        <v>96.75656827501791</v>
+        <v>96.7088660075274</v>
       </c>
     </row>
     <row r="41">
@@ -3983,19 +3983,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>27.55634918610405</v>
+        <v>25.55634918610405</v>
       </c>
       <c r="D41" t="n">
         <v>52.52691193458119</v>
       </c>
       <c r="E41" t="n">
-        <v>110.3259018078045</v>
+        <v>104.8111831820431</v>
       </c>
       <c r="F41" t="n">
-        <v>219.5807358037436</v>
+        <v>209.3797256769669</v>
       </c>
       <c r="G41" t="n">
-        <v>102.4974746830583</v>
+        <v>98.0685424949238</v>
       </c>
     </row>
     <row r="42">
@@ -4033,19 +4033,19 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>24.41811047550525</v>
+        <v>24.41488446708389</v>
       </c>
       <c r="D43" t="n">
-        <v>49.04921408900104</v>
+        <v>49.03946295574199</v>
       </c>
       <c r="E43" t="n">
-        <v>103.7222775834009</v>
+        <v>98.78888910980251</v>
       </c>
       <c r="F43" t="n">
-        <v>207.7440267546941</v>
+        <v>198.4048488856638</v>
       </c>
       <c r="G43" t="n">
-        <v>96.23340722565031</v>
+        <v>92.66202135457306</v>
       </c>
     </row>
     <row r="44">
@@ -4058,19 +4058,19 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>23.74064110506006</v>
+        <v>26.59251907515131</v>
       </c>
       <c r="D44" t="n">
-        <v>51.45450616521079</v>
+        <v>52.12313371305741</v>
       </c>
       <c r="E44" t="n">
-        <v>103.46142082518</v>
+        <v>104.9597785194129</v>
       </c>
       <c r="F44" t="n">
-        <v>207.7489479300626</v>
+        <v>210.8970608595957</v>
       </c>
       <c r="G44" t="n">
-        <v>96.60137900637835</v>
+        <v>98.6431230418043</v>
       </c>
     </row>
     <row r="45">
@@ -4108,19 +4108,19 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>24.83719391510835</v>
+        <v>25.71936168599622</v>
       </c>
       <c r="D46" t="n">
-        <v>51.45450616521079</v>
+        <v>52.12313371305741</v>
       </c>
       <c r="E46" t="n">
-        <v>103.46142082518</v>
+        <v>104.9597785194129</v>
       </c>
       <c r="F46" t="n">
-        <v>207.7489479300626</v>
+        <v>210.8970608595957</v>
       </c>
       <c r="G46" t="n">
-        <v>96.87551720889043</v>
+        <v>98.42483369451554</v>
       </c>
     </row>
     <row r="47">
@@ -4133,19 +4133,19 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>24.83719391510835</v>
+        <v>25.71936168599622</v>
       </c>
       <c r="D47" t="n">
-        <v>51.95837796962023</v>
+        <v>52.62700551746683</v>
       </c>
       <c r="E47" t="n">
-        <v>104.4691644339988</v>
+        <v>105.9675221282317</v>
       </c>
       <c r="F47" t="n">
-        <v>209.6068123063317</v>
+        <v>212.7549252358647</v>
       </c>
       <c r="G47" t="n">
-        <v>97.71788715626477</v>
+        <v>99.26720364188988</v>
       </c>
     </row>
     <row r="48">
@@ -4158,19 +4158,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>26.07297705925549</v>
+        <v>24.41488446708389</v>
       </c>
       <c r="D48" t="n">
-        <v>49.24441272425872</v>
+        <v>49.21635711250729</v>
       </c>
       <c r="E48" t="n">
-        <v>103.8198470130748</v>
+        <v>98.78888910980251</v>
       </c>
       <c r="F48" t="n">
-        <v>207.8890363034826</v>
+        <v>198.4048488856638</v>
       </c>
       <c r="G48" t="n">
-        <v>96.75656827501791</v>
+        <v>92.70624489376438</v>
       </c>
     </row>
     <row r="49">
@@ -4183,19 +4183,19 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>24.83719391510835</v>
+        <v>25.71936168599622</v>
       </c>
       <c r="D49" t="n">
-        <v>51.45450616521079</v>
+        <v>52.12313371305741</v>
       </c>
       <c r="E49" t="n">
-        <v>103.46142082518</v>
+        <v>104.9597785194129</v>
       </c>
       <c r="F49" t="n">
-        <v>207.7489479300626</v>
+        <v>210.8970608595957</v>
       </c>
       <c r="G49" t="n">
-        <v>96.87551720889043</v>
+        <v>98.42483369451554</v>
       </c>
     </row>
   </sheetData>
@@ -4309,19 +4309,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D4" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E4" t="n">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="F4" t="n">
-        <v>671</v>
+        <v>606</v>
       </c>
       <c r="G4" t="n">
-        <v>268.5</v>
+        <v>252.75</v>
       </c>
     </row>
     <row r="5">
@@ -4434,19 +4434,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D9" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E9" t="n">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="F9" t="n">
-        <v>631</v>
+        <v>616</v>
       </c>
       <c r="G9" t="n">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="10">
@@ -4534,19 +4534,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D13" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E13" t="n">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="F13" t="n">
-        <v>671</v>
+        <v>606</v>
       </c>
       <c r="G13" t="n">
-        <v>268.5</v>
+        <v>252.75</v>
       </c>
     </row>
     <row r="14">
@@ -4559,19 +4559,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D14" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="E14" t="n">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="F14" t="n">
-        <v>673</v>
+        <v>628</v>
       </c>
       <c r="G14" t="n">
-        <v>272.25</v>
+        <v>253</v>
       </c>
     </row>
     <row r="15">
@@ -4584,19 +4584,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D15" t="n">
         <v>90</v>
       </c>
       <c r="E15" t="n">
-        <v>225</v>
+        <v>211</v>
       </c>
       <c r="F15" t="n">
-        <v>497</v>
+        <v>455</v>
       </c>
       <c r="G15" t="n">
-        <v>210.75</v>
+        <v>196.25</v>
       </c>
     </row>
     <row r="16">
@@ -4684,19 +4684,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D19" t="n">
+        <v>12</v>
+      </c>
+      <c r="E19" t="n">
         <v>13</v>
       </c>
-      <c r="E19" t="n">
-        <v>15</v>
-      </c>
       <c r="F19" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G19" t="n">
-        <v>13.5</v>
+        <v>12.75</v>
       </c>
     </row>
     <row r="20">
@@ -4784,19 +4784,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D23" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E23" t="n">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="F23" t="n">
-        <v>631</v>
+        <v>616</v>
       </c>
       <c r="G23" t="n">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="24">
@@ -4812,16 +4812,16 @@
         <v>34</v>
       </c>
       <c r="D24" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E24" t="n">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="F24" t="n">
-        <v>581</v>
+        <v>508</v>
       </c>
       <c r="G24" t="n">
-        <v>237</v>
+        <v>220.75</v>
       </c>
     </row>
     <row r="25">
@@ -4834,19 +4834,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D25" t="n">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="E25" t="n">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F25" t="n">
-        <v>452</v>
+        <v>475</v>
       </c>
       <c r="G25" t="n">
-        <v>207.75</v>
+        <v>207.25</v>
       </c>
     </row>
     <row r="26">
@@ -4934,19 +4934,19 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D29" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="E29" t="n">
-        <v>283</v>
+        <v>256</v>
       </c>
       <c r="F29" t="n">
-        <v>673</v>
+        <v>628</v>
       </c>
       <c r="G29" t="n">
-        <v>272.25</v>
+        <v>253</v>
       </c>
     </row>
     <row r="30">
@@ -4959,19 +4959,19 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D30" t="n">
         <v>90</v>
       </c>
       <c r="E30" t="n">
-        <v>225</v>
+        <v>211</v>
       </c>
       <c r="F30" t="n">
-        <v>497</v>
+        <v>455</v>
       </c>
       <c r="G30" t="n">
-        <v>210.75</v>
+        <v>196.25</v>
       </c>
     </row>
     <row r="31">
@@ -4984,19 +4984,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D31" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E31" t="n">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="F31" t="n">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="G31" t="n">
-        <v>223.75</v>
+        <v>221.5</v>
       </c>
     </row>
     <row r="32">
@@ -5043,10 +5043,10 @@
         <v>17</v>
       </c>
       <c r="F33" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G33" t="n">
-        <v>16.25</v>
+        <v>15.75</v>
       </c>
     </row>
     <row r="34">
@@ -5109,19 +5109,19 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D36" t="n">
+        <v>12</v>
+      </c>
+      <c r="E36" t="n">
         <v>13</v>
       </c>
-      <c r="E36" t="n">
-        <v>15</v>
-      </c>
       <c r="F36" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G36" t="n">
-        <v>13.5</v>
+        <v>12.75</v>
       </c>
     </row>
     <row r="37">
@@ -5140,13 +5140,13 @@
         <v>13</v>
       </c>
       <c r="E37" t="n">
+        <v>11</v>
+      </c>
+      <c r="F37" t="n">
         <v>12</v>
       </c>
-      <c r="F37" t="n">
-        <v>13</v>
-      </c>
       <c r="G37" t="n">
-        <v>12.5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="38">
@@ -5187,16 +5187,16 @@
         <v>34</v>
       </c>
       <c r="D39" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E39" t="n">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="F39" t="n">
-        <v>581</v>
+        <v>508</v>
       </c>
       <c r="G39" t="n">
-        <v>237</v>
+        <v>220.75</v>
       </c>
     </row>
     <row r="40">
@@ -5209,19 +5209,19 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D40" t="n">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="E40" t="n">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F40" t="n">
-        <v>452</v>
+        <v>475</v>
       </c>
       <c r="G40" t="n">
-        <v>207.75</v>
+        <v>207.25</v>
       </c>
     </row>
     <row r="41">
@@ -5234,19 +5234,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D41" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="E41" t="n">
-        <v>260</v>
+        <v>279</v>
       </c>
       <c r="F41" t="n">
-        <v>518</v>
+        <v>605</v>
       </c>
       <c r="G41" t="n">
-        <v>231</v>
+        <v>259.5</v>
       </c>
     </row>
     <row r="42">
@@ -5284,19 +5284,19 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D43" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E43" t="n">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="F43" t="n">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="G43" t="n">
-        <v>223.75</v>
+        <v>221.5</v>
       </c>
     </row>
     <row r="44">
@@ -5318,10 +5318,10 @@
         <v>17</v>
       </c>
       <c r="F44" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G44" t="n">
-        <v>16.25</v>
+        <v>15.75</v>
       </c>
     </row>
     <row r="45">
@@ -5340,13 +5340,13 @@
         <v>20</v>
       </c>
       <c r="E45" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F45" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G45" t="n">
-        <v>17.5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="46">
@@ -5390,13 +5390,13 @@
         <v>13</v>
       </c>
       <c r="E47" t="n">
+        <v>11</v>
+      </c>
+      <c r="F47" t="n">
         <v>12</v>
       </c>
-      <c r="F47" t="n">
-        <v>13</v>
-      </c>
       <c r="G47" t="n">
-        <v>12.5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="48">
@@ -5409,19 +5409,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D48" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="E48" t="n">
-        <v>260</v>
+        <v>279</v>
       </c>
       <c r="F48" t="n">
-        <v>518</v>
+        <v>605</v>
       </c>
       <c r="G48" t="n">
-        <v>231</v>
+        <v>259.5</v>
       </c>
     </row>
     <row r="49">
@@ -5440,13 +5440,13 @@
         <v>20</v>
       </c>
       <c r="E49" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F49" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G49" t="n">
-        <v>17.5</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -5560,19 +5560,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D4" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="E4" t="n">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="F4" t="n">
-        <v>2280</v>
+        <v>2113</v>
       </c>
       <c r="G4" t="n">
-        <v>703.5</v>
+        <v>646.75</v>
       </c>
     </row>
     <row r="5">
@@ -5688,16 +5688,16 @@
         <v>41</v>
       </c>
       <c r="D9" t="n">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E9" t="n">
-        <v>496</v>
+        <v>463</v>
       </c>
       <c r="F9" t="n">
-        <v>1909</v>
+        <v>1824</v>
       </c>
       <c r="G9" t="n">
-        <v>644</v>
+        <v>613</v>
       </c>
     </row>
     <row r="10">
@@ -5785,19 +5785,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D13" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="E13" t="n">
-        <v>410</v>
+        <v>365</v>
       </c>
       <c r="F13" t="n">
-        <v>2280</v>
+        <v>2113</v>
       </c>
       <c r="G13" t="n">
-        <v>703.5</v>
+        <v>646.75</v>
       </c>
     </row>
     <row r="14">
@@ -5810,19 +5810,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D14" t="n">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E14" t="n">
-        <v>410</v>
+        <v>353</v>
       </c>
       <c r="F14" t="n">
-        <v>2242</v>
+        <v>2096</v>
       </c>
       <c r="G14" t="n">
-        <v>694</v>
+        <v>639.75</v>
       </c>
     </row>
     <row r="15">
@@ -5835,19 +5835,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D15" t="n">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="E15" t="n">
-        <v>525</v>
+        <v>478</v>
       </c>
       <c r="F15" t="n">
-        <v>2852</v>
+        <v>2444</v>
       </c>
       <c r="G15" t="n">
-        <v>881.5</v>
+        <v>767.75</v>
       </c>
     </row>
     <row r="16">
@@ -5935,19 +5935,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D19" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E19" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="F19" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G19" t="n">
-        <v>34</v>
+        <v>31.25</v>
       </c>
     </row>
     <row r="20">
@@ -6038,16 +6038,16 @@
         <v>41</v>
       </c>
       <c r="D23" t="n">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E23" t="n">
-        <v>496</v>
+        <v>463</v>
       </c>
       <c r="F23" t="n">
-        <v>1909</v>
+        <v>1824</v>
       </c>
       <c r="G23" t="n">
-        <v>644</v>
+        <v>613</v>
       </c>
     </row>
     <row r="24">
@@ -6060,19 +6060,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D24" t="n">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="E24" t="n">
-        <v>526</v>
+        <v>478</v>
       </c>
       <c r="F24" t="n">
-        <v>2111</v>
+        <v>1954</v>
       </c>
       <c r="G24" t="n">
-        <v>703.25</v>
+        <v>650</v>
       </c>
     </row>
     <row r="25">
@@ -6085,19 +6085,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D25" t="n">
-        <v>186</v>
+        <v>161</v>
       </c>
       <c r="E25" t="n">
-        <v>645</v>
+        <v>605</v>
       </c>
       <c r="F25" t="n">
-        <v>2471</v>
+        <v>2384</v>
       </c>
       <c r="G25" t="n">
-        <v>836.75</v>
+        <v>800</v>
       </c>
     </row>
     <row r="26">
@@ -6185,19 +6185,19 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D29" t="n">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="E29" t="n">
-        <v>410</v>
+        <v>353</v>
       </c>
       <c r="F29" t="n">
-        <v>2242</v>
+        <v>2096</v>
       </c>
       <c r="G29" t="n">
-        <v>694</v>
+        <v>639.75</v>
       </c>
     </row>
     <row r="30">
@@ -6210,19 +6210,19 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D30" t="n">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="E30" t="n">
-        <v>525</v>
+        <v>478</v>
       </c>
       <c r="F30" t="n">
-        <v>2852</v>
+        <v>2444</v>
       </c>
       <c r="G30" t="n">
-        <v>881.5</v>
+        <v>767.75</v>
       </c>
     </row>
     <row r="31">
@@ -6235,19 +6235,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D31" t="n">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="E31" t="n">
-        <v>529</v>
+        <v>454</v>
       </c>
       <c r="F31" t="n">
-        <v>2864</v>
+        <v>2132</v>
       </c>
       <c r="G31" t="n">
-        <v>886.25</v>
+        <v>683.25</v>
       </c>
     </row>
     <row r="32">
@@ -6285,19 +6285,19 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D33" t="n">
         <v>38</v>
       </c>
       <c r="E33" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F33" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G33" t="n">
-        <v>36.25</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="34">
@@ -6360,19 +6360,19 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D36" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E36" t="n">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="F36" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G36" t="n">
-        <v>34</v>
+        <v>31.25</v>
       </c>
     </row>
     <row r="37">
@@ -6388,16 +6388,16 @@
         <v>20</v>
       </c>
       <c r="D37" t="n">
+        <v>33</v>
+      </c>
+      <c r="E37" t="n">
+        <v>33</v>
+      </c>
+      <c r="F37" t="n">
         <v>38</v>
       </c>
-      <c r="E37" t="n">
-        <v>37</v>
-      </c>
-      <c r="F37" t="n">
-        <v>45</v>
-      </c>
       <c r="G37" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="38">
@@ -6435,19 +6435,19 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D39" t="n">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="E39" t="n">
-        <v>526</v>
+        <v>478</v>
       </c>
       <c r="F39" t="n">
-        <v>2111</v>
+        <v>1954</v>
       </c>
       <c r="G39" t="n">
-        <v>703.25</v>
+        <v>650</v>
       </c>
     </row>
     <row r="40">
@@ -6460,19 +6460,19 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D40" t="n">
-        <v>186</v>
+        <v>161</v>
       </c>
       <c r="E40" t="n">
-        <v>645</v>
+        <v>605</v>
       </c>
       <c r="F40" t="n">
-        <v>2471</v>
+        <v>2384</v>
       </c>
       <c r="G40" t="n">
-        <v>836.75</v>
+        <v>800</v>
       </c>
     </row>
     <row r="41">
@@ -6485,19 +6485,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="D41" t="n">
-        <v>194</v>
+        <v>177</v>
       </c>
       <c r="E41" t="n">
-        <v>697</v>
+        <v>657</v>
       </c>
       <c r="F41" t="n">
-        <v>2585</v>
+        <v>2515</v>
       </c>
       <c r="G41" t="n">
-        <v>881.5</v>
+        <v>851.75</v>
       </c>
     </row>
     <row r="42">
@@ -6535,19 +6535,19 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D43" t="n">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="E43" t="n">
-        <v>529</v>
+        <v>454</v>
       </c>
       <c r="F43" t="n">
-        <v>2864</v>
+        <v>2132</v>
       </c>
       <c r="G43" t="n">
-        <v>886.25</v>
+        <v>683.25</v>
       </c>
     </row>
     <row r="44">
@@ -6560,19 +6560,19 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D44" t="n">
         <v>38</v>
       </c>
       <c r="E44" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F44" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G44" t="n">
-        <v>36.25</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="45">
@@ -6588,16 +6588,16 @@
         <v>23</v>
       </c>
       <c r="D45" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E45" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F45" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G45" t="n">
-        <v>38.25</v>
+        <v>35.75</v>
       </c>
     </row>
     <row r="46">
@@ -6638,16 +6638,16 @@
         <v>20</v>
       </c>
       <c r="D47" t="n">
+        <v>33</v>
+      </c>
+      <c r="E47" t="n">
+        <v>33</v>
+      </c>
+      <c r="F47" t="n">
         <v>38</v>
       </c>
-      <c r="E47" t="n">
-        <v>37</v>
-      </c>
-      <c r="F47" t="n">
-        <v>45</v>
-      </c>
       <c r="G47" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="48">
@@ -6660,19 +6660,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="D48" t="n">
-        <v>194</v>
+        <v>177</v>
       </c>
       <c r="E48" t="n">
-        <v>697</v>
+        <v>657</v>
       </c>
       <c r="F48" t="n">
-        <v>2585</v>
+        <v>2515</v>
       </c>
       <c r="G48" t="n">
-        <v>881.5</v>
+        <v>851.75</v>
       </c>
     </row>
     <row r="49">
@@ -6688,16 +6688,16 @@
         <v>23</v>
       </c>
       <c r="D49" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E49" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F49" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G49" t="n">
-        <v>38.25</v>
+        <v>35.75</v>
       </c>
     </row>
   </sheetData>
@@ -6814,16 +6814,16 @@
         <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F4" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G4" t="n">
-        <v>16.75</v>
+        <v>16.25</v>
       </c>
     </row>
     <row r="5">
@@ -6936,19 +6936,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D9" t="n">
         <v>14</v>
       </c>
       <c r="E9" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F9" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G9" t="n">
-        <v>15</v>
+        <v>14.25</v>
       </c>
     </row>
     <row r="10">
@@ -7036,7 +7036,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D13" t="n">
         <v>6</v>
@@ -7048,7 +7048,7 @@
         <v>7</v>
       </c>
       <c r="G13" t="n">
-        <v>6.75</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="14">
@@ -7061,7 +7061,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D14" t="n">
         <v>12</v>
@@ -7073,7 +7073,7 @@
         <v>18</v>
       </c>
       <c r="G14" t="n">
-        <v>13.5</v>
+        <v>13.75</v>
       </c>
     </row>
     <row r="15">
@@ -7086,19 +7086,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D15" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E15" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F15" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="G15" t="n">
-        <v>13.5</v>
+        <v>18.75</v>
       </c>
     </row>
     <row r="16">
@@ -7186,19 +7186,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D19" t="n">
         <v>13</v>
       </c>
       <c r="E19" t="n">
+        <v>13</v>
+      </c>
+      <c r="F19" t="n">
         <v>15</v>
       </c>
-      <c r="F19" t="n">
-        <v>13</v>
-      </c>
       <c r="G19" t="n">
-        <v>13.25</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="20">
@@ -7236,19 +7236,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G21" t="n">
-        <v>6.5</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="22">
@@ -7311,7 +7311,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D24" t="n">
         <v>11</v>
@@ -7323,7 +7323,7 @@
         <v>12</v>
       </c>
       <c r="G24" t="n">
-        <v>12</v>
+        <v>12.25</v>
       </c>
     </row>
     <row r="25">
@@ -7336,19 +7336,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D25" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E25" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F25" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="G25" t="n">
-        <v>16.75</v>
+        <v>21</v>
       </c>
     </row>
     <row r="26">
@@ -7461,10 +7461,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D30" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E30" t="n">
         <v>7</v>
@@ -7473,7 +7473,7 @@
         <v>7</v>
       </c>
       <c r="G30" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="31">
@@ -7486,19 +7486,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D31" t="n">
         <v>12</v>
       </c>
       <c r="E31" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F31" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G31" t="n">
-        <v>13.5</v>
+        <v>11.75</v>
       </c>
     </row>
     <row r="32">
@@ -7536,7 +7536,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D33" t="n">
         <v>14</v>
@@ -7548,7 +7548,7 @@
         <v>14</v>
       </c>
       <c r="G33" t="n">
-        <v>13.25</v>
+        <v>13.75</v>
       </c>
     </row>
     <row r="34">
@@ -7586,19 +7586,19 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D35" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E35" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F35" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G35" t="n">
-        <v>5.75</v>
+        <v>6.75</v>
       </c>
     </row>
     <row r="36">
@@ -7611,19 +7611,19 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D36" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E36" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F36" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G36" t="n">
-        <v>8.5</v>
+        <v>9.75</v>
       </c>
     </row>
     <row r="37">
@@ -7661,19 +7661,19 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D38" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E38" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F38" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G38" t="n">
-        <v>6.25</v>
+        <v>7.25</v>
       </c>
     </row>
     <row r="39">
@@ -7714,7 +7714,7 @@
         <v>7</v>
       </c>
       <c r="D40" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E40" t="n">
         <v>8</v>
@@ -7723,7 +7723,7 @@
         <v>8</v>
       </c>
       <c r="G40" t="n">
-        <v>7.5</v>
+        <v>7.75</v>
       </c>
     </row>
     <row r="41">
@@ -7736,19 +7736,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D41" t="n">
         <v>13</v>
       </c>
       <c r="E41" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F41" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G41" t="n">
-        <v>16.25</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="42">
@@ -7786,19 +7786,19 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D43" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E43" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F43" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G43" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44">
@@ -7811,19 +7811,19 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D44" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E44" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F44" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G44" t="n">
-        <v>6.75</v>
+        <v>8.25</v>
       </c>
     </row>
     <row r="45">
@@ -7861,19 +7861,19 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D46" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E46" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F46" t="n">
+        <v>9</v>
+      </c>
+      <c r="G46" t="n">
         <v>8</v>
-      </c>
-      <c r="G46" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="47">
@@ -7886,19 +7886,19 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G47" t="n">
-        <v>7.5</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="48">
@@ -7911,19 +7911,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D48" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E48" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F48" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G48" t="n">
-        <v>7.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="49">
@@ -7936,19 +7936,19 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D49" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E49" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F49" t="n">
+        <v>9</v>
+      </c>
+      <c r="G49" t="n">
         <v>8</v>
-      </c>
-      <c r="G49" t="n">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -8037,16 +8037,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C4" t="n">
-        <v>193</v>
+        <v>177</v>
       </c>
       <c r="D4" t="n">
-        <v>684</v>
+        <v>641</v>
       </c>
       <c r="E4" t="n">
-        <v>2951</v>
+        <v>2719</v>
       </c>
     </row>
     <row r="5">
@@ -8132,16 +8132,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C9" t="n">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="D9" t="n">
-        <v>774</v>
+        <v>750</v>
       </c>
       <c r="E9" t="n">
-        <v>2540</v>
+        <v>2440</v>
       </c>
     </row>
     <row r="10">
@@ -8208,16 +8208,16 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C13" t="n">
-        <v>193</v>
+        <v>177</v>
       </c>
       <c r="D13" t="n">
-        <v>684</v>
+        <v>641</v>
       </c>
       <c r="E13" t="n">
-        <v>2951</v>
+        <v>2719</v>
       </c>
     </row>
     <row r="14">
@@ -8227,16 +8227,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C14" t="n">
-        <v>194</v>
+        <v>176</v>
       </c>
       <c r="D14" t="n">
-        <v>693</v>
+        <v>609</v>
       </c>
       <c r="E14" t="n">
-        <v>2915</v>
+        <v>2724</v>
       </c>
     </row>
     <row r="15">
@@ -8246,16 +8246,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C15" t="n">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="D15" t="n">
-        <v>750</v>
+        <v>689</v>
       </c>
       <c r="E15" t="n">
-        <v>3349</v>
+        <v>2899</v>
       </c>
     </row>
     <row r="16">
@@ -8322,16 +8322,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C19" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D19" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E19" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20">
@@ -8398,16 +8398,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C23" t="n">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="D23" t="n">
-        <v>774</v>
+        <v>750</v>
       </c>
       <c r="E23" t="n">
-        <v>2540</v>
+        <v>2440</v>
       </c>
     </row>
     <row r="24">
@@ -8417,16 +8417,16 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C24" t="n">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="D24" t="n">
-        <v>766</v>
+        <v>727</v>
       </c>
       <c r="E24" t="n">
-        <v>2692</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="25">
@@ -8439,13 +8439,13 @@
         <v>80</v>
       </c>
       <c r="C25" t="n">
-        <v>301</v>
+        <v>255</v>
       </c>
       <c r="D25" t="n">
-        <v>874</v>
+        <v>835</v>
       </c>
       <c r="E25" t="n">
-        <v>2923</v>
+        <v>2859</v>
       </c>
     </row>
     <row r="26">
@@ -8512,16 +8512,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C29" t="n">
-        <v>194</v>
+        <v>176</v>
       </c>
       <c r="D29" t="n">
-        <v>693</v>
+        <v>609</v>
       </c>
       <c r="E29" t="n">
-        <v>2915</v>
+        <v>2724</v>
       </c>
     </row>
     <row r="30">
@@ -8531,16 +8531,16 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C30" t="n">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="D30" t="n">
-        <v>750</v>
+        <v>689</v>
       </c>
       <c r="E30" t="n">
-        <v>3349</v>
+        <v>2899</v>
       </c>
     </row>
     <row r="31">
@@ -8550,16 +8550,16 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C31" t="n">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="D31" t="n">
-        <v>771</v>
+        <v>688</v>
       </c>
       <c r="E31" t="n">
-        <v>3397</v>
+        <v>2663</v>
       </c>
     </row>
     <row r="32">
@@ -8588,16 +8588,16 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C33" t="n">
         <v>55</v>
       </c>
       <c r="D33" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E33" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="34">
@@ -8645,16 +8645,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C36" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D36" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E36" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="37">
@@ -8667,13 +8667,13 @@
         <v>32</v>
       </c>
       <c r="C37" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D37" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E37" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="38">
@@ -8702,16 +8702,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C39" t="n">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="D39" t="n">
-        <v>766</v>
+        <v>727</v>
       </c>
       <c r="E39" t="n">
-        <v>2692</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="40">
@@ -8724,13 +8724,13 @@
         <v>80</v>
       </c>
       <c r="C40" t="n">
-        <v>301</v>
+        <v>255</v>
       </c>
       <c r="D40" t="n">
-        <v>874</v>
+        <v>835</v>
       </c>
       <c r="E40" t="n">
-        <v>2923</v>
+        <v>2859</v>
       </c>
     </row>
     <row r="41">
@@ -8740,16 +8740,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="C41" t="n">
-        <v>308</v>
+        <v>295</v>
       </c>
       <c r="D41" t="n">
-        <v>957</v>
+        <v>936</v>
       </c>
       <c r="E41" t="n">
-        <v>3103</v>
+        <v>3120</v>
       </c>
     </row>
     <row r="42">
@@ -8778,16 +8778,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C43" t="n">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="D43" t="n">
-        <v>771</v>
+        <v>688</v>
       </c>
       <c r="E43" t="n">
-        <v>3397</v>
+        <v>2663</v>
       </c>
     </row>
     <row r="44">
@@ -8797,16 +8797,16 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C44" t="n">
         <v>55</v>
       </c>
       <c r="D44" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E44" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45">
@@ -8819,13 +8819,13 @@
         <v>36</v>
       </c>
       <c r="C45" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D45" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E45" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="46">
@@ -8857,13 +8857,13 @@
         <v>32</v>
       </c>
       <c r="C47" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D47" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E47" t="n">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="48">
@@ -8873,16 +8873,16 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="C48" t="n">
-        <v>308</v>
+        <v>295</v>
       </c>
       <c r="D48" t="n">
-        <v>957</v>
+        <v>936</v>
       </c>
       <c r="E48" t="n">
-        <v>3103</v>
+        <v>3120</v>
       </c>
     </row>
     <row r="49">
@@ -8895,13 +8895,13 @@
         <v>36</v>
       </c>
       <c r="C49" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D49" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E49" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
checkout untuk fix ouput perhitungan manual
</commit_message>
<xml_diff>
--- a/Excel/Validasi/Hasil_Pengujian_Map_1_128_avg_length.xlsx
+++ b/Excel/Validasi/Hasil_Pengujian_Map_1_128_avg_length.xlsx
@@ -506,19 +506,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.000488</v>
+        <v>0.0004585</v>
       </c>
       <c r="D2" t="n">
-        <v>0.002934</v>
+        <v>0.0028168</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0191111</v>
+        <v>0.0190411</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1264418</v>
+        <v>0.121997</v>
       </c>
       <c r="G2" t="n">
-        <v>0.037243725</v>
+        <v>0.03607835</v>
       </c>
     </row>
     <row r="3">
@@ -531,19 +531,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.0003022</v>
+        <v>0.0003069</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0011951</v>
+        <v>0.0012239</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0049929</v>
+        <v>0.0048175</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0208262</v>
+        <v>0.0200653</v>
       </c>
       <c r="G3" t="n">
-        <v>0.006829100000000001</v>
+        <v>0.006603400000000001</v>
       </c>
     </row>
     <row r="4">
@@ -556,19 +556,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.0004053</v>
+        <v>0.0005399</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0018053</v>
+        <v>0.0018485</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0142213</v>
+        <v>0.0163242</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1646243</v>
+        <v>0.1526633</v>
       </c>
       <c r="G4" t="n">
-        <v>0.04526405</v>
+        <v>0.042843975</v>
       </c>
     </row>
     <row r="5">
@@ -581,19 +581,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.0003970999999999999</v>
+        <v>0.0003932</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0023637</v>
+        <v>0.0023093</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0155513</v>
+        <v>0.0154216</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1113312</v>
+        <v>0.1059115</v>
       </c>
       <c r="G5" t="n">
-        <v>0.032410825</v>
+        <v>0.0310089</v>
       </c>
     </row>
     <row r="6">
@@ -606,19 +606,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.0003778</v>
+        <v>0.0003333</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0009717</v>
+        <v>0.0009808</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0033759</v>
+        <v>0.003392399999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>0.012292</v>
+        <v>0.0122929</v>
       </c>
       <c r="G6" t="n">
-        <v>0.00425435</v>
+        <v>0.004249849999999999</v>
       </c>
     </row>
     <row r="7">
@@ -631,19 +631,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.0006016000000000001</v>
+        <v>0.000512</v>
       </c>
       <c r="D7" t="n">
-        <v>0.003082</v>
+        <v>0.0029314</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0195018</v>
+        <v>0.0183713</v>
       </c>
       <c r="F7" t="n">
-        <v>0.127873</v>
+        <v>0.1215531</v>
       </c>
       <c r="G7" t="n">
-        <v>0.0377646</v>
+        <v>0.03584195</v>
       </c>
     </row>
     <row r="8">
@@ -656,19 +656,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.0005254999999999999</v>
+        <v>0.000531</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0027902</v>
+        <v>0.0027971</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0178527</v>
+        <v>0.017198</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1198106</v>
+        <v>0.117049</v>
       </c>
       <c r="G8" t="n">
-        <v>0.03524475</v>
+        <v>0.034393775</v>
       </c>
     </row>
     <row r="9">
@@ -681,19 +681,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.0004429</v>
+        <v>0.0004536999999999999</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0016992</v>
+        <v>0.0019769</v>
       </c>
       <c r="E9" t="n">
-        <v>0.008820700000000001</v>
+        <v>0.0121841</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0528004</v>
+        <v>0.08451460000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0159408</v>
+        <v>0.024782325</v>
       </c>
     </row>
     <row r="10">
@@ -706,19 +706,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.0003189</v>
+        <v>0.0003224</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0013871</v>
+        <v>0.001383</v>
       </c>
       <c r="E10" t="n">
-        <v>0.005935</v>
+        <v>0.0057414</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0249958</v>
+        <v>0.024999</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0081592</v>
+        <v>0.008111449999999999</v>
       </c>
     </row>
     <row r="11">
@@ -731,19 +731,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.0003365</v>
+        <v>0.0003191</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0013536</v>
+        <v>0.0013039</v>
       </c>
       <c r="E11" t="n">
-        <v>0.005054500000000001</v>
+        <v>0.0051039</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0217027</v>
+        <v>0.0209627</v>
       </c>
       <c r="G11" t="n">
-        <v>0.007111825</v>
+        <v>0.0069224</v>
       </c>
     </row>
     <row r="12">
@@ -756,19 +756,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.0003193</v>
+        <v>0.0003317</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0014867</v>
+        <v>0.0014245</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0054447</v>
+        <v>0.005322</v>
       </c>
       <c r="F12" t="n">
-        <v>0.021916</v>
+        <v>0.0213904</v>
       </c>
       <c r="G12" t="n">
-        <v>0.007291674999999999</v>
+        <v>0.00711715</v>
       </c>
     </row>
     <row r="13">
@@ -781,19 +781,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.0004682000000000001</v>
+        <v>0.0005563</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0019299</v>
+        <v>0.0020061</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0142374</v>
+        <v>0.0168071</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1669026</v>
+        <v>0.1526683</v>
       </c>
       <c r="G13" t="n">
-        <v>0.045884525</v>
+        <v>0.04300945</v>
       </c>
     </row>
     <row r="14">
@@ -806,19 +806,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.0004872</v>
+        <v>0.0005176</v>
       </c>
       <c r="D14" t="n">
-        <v>0.001915</v>
+        <v>0.001937</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0138306</v>
+        <v>0.0183092</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1616847</v>
+        <v>0.1633502</v>
       </c>
       <c r="G14" t="n">
-        <v>0.04447937499999999</v>
+        <v>0.0460285</v>
       </c>
     </row>
     <row r="15">
@@ -831,19 +831,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.0005844</v>
+        <v>0.0005661</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0026095</v>
+        <v>0.0025919</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0183228</v>
+        <v>0.0192865</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1764387</v>
+        <v>0.1745935</v>
       </c>
       <c r="G15" t="n">
-        <v>0.04948885</v>
+        <v>0.0492595</v>
       </c>
     </row>
     <row r="16">
@@ -856,19 +856,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.0004614</v>
+        <v>0.0004626</v>
       </c>
       <c r="D16" t="n">
-        <v>0.00241</v>
+        <v>0.0023947</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0156817</v>
+        <v>0.0154221</v>
       </c>
       <c r="F16" t="n">
-        <v>0.1132413</v>
+        <v>0.1068417</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0329486</v>
+        <v>0.031280275</v>
       </c>
     </row>
     <row r="17">
@@ -881,19 +881,19 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.0005739</v>
+        <v>0.0005595</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0035986</v>
+        <v>0.0033448</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0158411</v>
+        <v>0.0153551</v>
       </c>
       <c r="F17" t="n">
-        <v>0.1056952</v>
+        <v>0.1014004</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0314272</v>
+        <v>0.03016495</v>
       </c>
     </row>
     <row r="18">
@@ -906,19 +906,19 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.0003591</v>
+        <v>0.0003228999999999999</v>
       </c>
       <c r="D18" t="n">
-        <v>0.00098</v>
+        <v>0.000915</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0028888</v>
+        <v>0.0028975</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0108466</v>
+        <v>0.010835</v>
       </c>
       <c r="G18" t="n">
-        <v>0.003768625</v>
+        <v>0.0037426</v>
       </c>
     </row>
     <row r="19">
@@ -931,19 +931,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.0003145</v>
+        <v>0.0003366</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0008716999999999999</v>
+        <v>0.0009219999999999999</v>
       </c>
       <c r="E19" t="n">
-        <v>0.0025937</v>
+        <v>0.0029943</v>
       </c>
       <c r="F19" t="n">
-        <v>0.0121766</v>
+        <v>0.0106857</v>
       </c>
       <c r="G19" t="n">
-        <v>0.003989125</v>
+        <v>0.00373465</v>
       </c>
     </row>
     <row r="20">
@@ -956,19 +956,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.000361</v>
+        <v>0.0003364999999999999</v>
       </c>
       <c r="D20" t="n">
-        <v>0.0011302</v>
+        <v>0.0010501</v>
       </c>
       <c r="E20" t="n">
-        <v>0.0036276</v>
+        <v>0.0036458</v>
       </c>
       <c r="F20" t="n">
-        <v>0.0133442</v>
+        <v>0.0131556</v>
       </c>
       <c r="G20" t="n">
-        <v>0.00461575</v>
+        <v>0.004547</v>
       </c>
     </row>
     <row r="21">
@@ -981,19 +981,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.0003751</v>
+        <v>0.0003587999999999999</v>
       </c>
       <c r="D21" t="n">
-        <v>0.0011003</v>
+        <v>0.0009927</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0034493</v>
+        <v>0.0033916</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0122192</v>
+        <v>0.0123284</v>
       </c>
       <c r="G21" t="n">
-        <v>0.004285975</v>
+        <v>0.004267874999999999</v>
       </c>
     </row>
     <row r="22">
@@ -1006,19 +1006,19 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.0005897000000000001</v>
+        <v>0.0005886999999999999</v>
       </c>
       <c r="D22" t="n">
-        <v>0.0029227</v>
+        <v>0.0028023</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0182536</v>
+        <v>0.0172376</v>
       </c>
       <c r="F22" t="n">
-        <v>0.1212913</v>
+        <v>0.117096</v>
       </c>
       <c r="G22" t="n">
-        <v>0.035764325</v>
+        <v>0.03443115</v>
       </c>
     </row>
     <row r="23">
@@ -1031,19 +1031,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.0005002</v>
+        <v>0.0004895</v>
       </c>
       <c r="D23" t="n">
-        <v>0.0017475</v>
+        <v>0.002076</v>
       </c>
       <c r="E23" t="n">
-        <v>0.008291099999999999</v>
+        <v>0.0126124</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0530564</v>
+        <v>0.0852088</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0158988</v>
+        <v>0.025096675</v>
       </c>
     </row>
     <row r="24">
@@ -1056,19 +1056,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.0005290999999999999</v>
+        <v>0.0005012</v>
       </c>
       <c r="D24" t="n">
-        <v>0.0017723</v>
+        <v>0.0021151</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0085497</v>
+        <v>0.0127391</v>
       </c>
       <c r="F24" t="n">
-        <v>0.0533539</v>
+        <v>0.08367049999999999</v>
       </c>
       <c r="G24" t="n">
-        <v>0.01605125</v>
+        <v>0.024756475</v>
       </c>
     </row>
     <row r="25">
@@ -1081,19 +1081,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.0005549</v>
+        <v>0.0005079000000000001</v>
       </c>
       <c r="D25" t="n">
-        <v>0.0023584</v>
+        <v>0.0026978</v>
       </c>
       <c r="E25" t="n">
-        <v>0.012572</v>
+        <v>0.0159835</v>
       </c>
       <c r="F25" t="n">
-        <v>0.0846522</v>
+        <v>0.1215122</v>
       </c>
       <c r="G25" t="n">
-        <v>0.025034375</v>
+        <v>0.03517535</v>
       </c>
     </row>
     <row r="26">
@@ -1106,19 +1106,19 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.0003788</v>
+        <v>0.0003762</v>
       </c>
       <c r="D26" t="n">
-        <v>0.0015154</v>
+        <v>0.0014629</v>
       </c>
       <c r="E26" t="n">
-        <v>0.006075</v>
+        <v>0.0073336</v>
       </c>
       <c r="F26" t="n">
-        <v>0.0262154</v>
+        <v>0.025562</v>
       </c>
       <c r="G26" t="n">
-        <v>0.008546149999999999</v>
+        <v>0.008683675</v>
       </c>
     </row>
     <row r="27">
@@ -1131,19 +1131,19 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.0003761</v>
+        <v>0.0003649</v>
       </c>
       <c r="D27" t="n">
-        <v>0.0016044</v>
+        <v>0.0016179</v>
       </c>
       <c r="E27" t="n">
-        <v>0.0063856</v>
+        <v>0.0062774</v>
       </c>
       <c r="F27" t="n">
-        <v>0.0264375</v>
+        <v>0.0266712</v>
       </c>
       <c r="G27" t="n">
-        <v>0.008700899999999999</v>
+        <v>0.008732849999999999</v>
       </c>
     </row>
     <row r="28">
@@ -1156,19 +1156,19 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.000369</v>
+        <v>0.0003608</v>
       </c>
       <c r="D28" t="n">
-        <v>0.0015119</v>
+        <v>0.0015419</v>
       </c>
       <c r="E28" t="n">
-        <v>0.005735599999999999</v>
+        <v>0.0055933</v>
       </c>
       <c r="F28" t="n">
-        <v>0.0228551</v>
+        <v>0.0221864</v>
       </c>
       <c r="G28" t="n">
-        <v>0.007617899999999999</v>
+        <v>0.007420599999999999</v>
       </c>
     </row>
     <row r="29">
@@ -1181,19 +1181,19 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.0005112000000000001</v>
+        <v>0.000537</v>
       </c>
       <c r="D29" t="n">
-        <v>0.0020943</v>
+        <v>0.0019312</v>
       </c>
       <c r="E29" t="n">
-        <v>0.0142882</v>
+        <v>0.0186731</v>
       </c>
       <c r="F29" t="n">
-        <v>0.1643884</v>
+        <v>0.1643973</v>
       </c>
       <c r="G29" t="n">
-        <v>0.045320525</v>
+        <v>0.04638465000000001</v>
       </c>
     </row>
     <row r="30">
@@ -1206,19 +1206,19 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.0006200999999999999</v>
+        <v>0.0005811999999999999</v>
       </c>
       <c r="D30" t="n">
-        <v>0.0025644</v>
+        <v>0.0026649</v>
       </c>
       <c r="E30" t="n">
-        <v>0.0187376</v>
+        <v>0.0201055</v>
       </c>
       <c r="F30" t="n">
-        <v>0.179151</v>
+        <v>0.1749841</v>
       </c>
       <c r="G30" t="n">
-        <v>0.050268275</v>
+        <v>0.04958392500000001</v>
       </c>
     </row>
     <row r="31">
@@ -1231,19 +1231,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.0006041</v>
+        <v>0.0005631</v>
       </c>
       <c r="D31" t="n">
-        <v>0.0027139</v>
+        <v>0.002918599999999999</v>
       </c>
       <c r="E31" t="n">
-        <v>0.0179335</v>
+        <v>0.0205008</v>
       </c>
       <c r="F31" t="n">
-        <v>0.1518734</v>
+        <v>0.1938393</v>
       </c>
       <c r="G31" t="n">
-        <v>0.043281225</v>
+        <v>0.05445545</v>
       </c>
     </row>
     <row r="32">
@@ -1256,19 +1256,19 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0.0006119</v>
+        <v>0.0006108000000000001</v>
       </c>
       <c r="D32" t="n">
-        <v>0.0035223</v>
+        <v>0.0033888</v>
       </c>
       <c r="E32" t="n">
-        <v>0.0160673</v>
+        <v>0.0156853</v>
       </c>
       <c r="F32" t="n">
-        <v>0.1078077</v>
+        <v>0.1025261</v>
       </c>
       <c r="G32" t="n">
-        <v>0.0320023</v>
+        <v>0.03055275</v>
       </c>
     </row>
     <row r="33">
@@ -1281,19 +1281,19 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0.0004094</v>
+        <v>0.0002847</v>
       </c>
       <c r="D33" t="n">
-        <v>0.0011284</v>
+        <v>0.0009162</v>
       </c>
       <c r="E33" t="n">
-        <v>0.0032717</v>
+        <v>0.002679400000000001</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0107584</v>
+        <v>0.0082586</v>
       </c>
       <c r="G33" t="n">
-        <v>0.003891975</v>
+        <v>0.003034725</v>
       </c>
     </row>
     <row r="34">
@@ -1306,19 +1306,19 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0.0003128000000000001</v>
+        <v>0.0002686</v>
       </c>
       <c r="D34" t="n">
-        <v>0.0010323</v>
+        <v>0.0009722999999999999</v>
       </c>
       <c r="E34" t="n">
-        <v>0.0029806</v>
+        <v>0.0029487</v>
       </c>
       <c r="F34" t="n">
-        <v>0.0113632</v>
+        <v>0.0110795</v>
       </c>
       <c r="G34" t="n">
-        <v>0.003922225000000001</v>
+        <v>0.003817275</v>
       </c>
     </row>
     <row r="35">
@@ -1331,19 +1331,19 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.0004091</v>
+        <v>0.0003697999999999999</v>
       </c>
       <c r="D35" t="n">
-        <v>0.0009947999999999999</v>
+        <v>0.0009679000000000001</v>
       </c>
       <c r="E35" t="n">
-        <v>0.0029447</v>
+        <v>0.0029392</v>
       </c>
       <c r="F35" t="n">
-        <v>0.0111221</v>
+        <v>0.0109433</v>
       </c>
       <c r="G35" t="n">
-        <v>0.003867675</v>
+        <v>0.00380505</v>
       </c>
     </row>
     <row r="36">
@@ -1356,19 +1356,19 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0.0003565</v>
+        <v>0.0003255</v>
       </c>
       <c r="D36" t="n">
-        <v>0.0009288999999999999</v>
+        <v>0.0009538000000000001</v>
       </c>
       <c r="E36" t="n">
-        <v>0.0025786</v>
+        <v>0.0030312</v>
       </c>
       <c r="F36" t="n">
-        <v>0.0121538</v>
+        <v>0.0109231</v>
       </c>
       <c r="G36" t="n">
-        <v>0.00400445</v>
+        <v>0.0038084</v>
       </c>
     </row>
     <row r="37">
@@ -1381,19 +1381,19 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0.000322</v>
+        <v>0.0003422</v>
       </c>
       <c r="D37" t="n">
-        <v>0.0009711000000000001</v>
+        <v>0.0010449</v>
       </c>
       <c r="E37" t="n">
-        <v>0.0026808</v>
+        <v>0.003267299999999999</v>
       </c>
       <c r="F37" t="n">
-        <v>0.0114559</v>
+        <v>0.0113351</v>
       </c>
       <c r="G37" t="n">
-        <v>0.00385745</v>
+        <v>0.003997374999999999</v>
       </c>
     </row>
     <row r="38">
@@ -1406,19 +1406,19 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0.0004107000000000001</v>
+        <v>0.0003655</v>
       </c>
       <c r="D38" t="n">
-        <v>0.0012051</v>
+        <v>0.0011678</v>
       </c>
       <c r="E38" t="n">
-        <v>0.0036779</v>
+        <v>0.0035601</v>
       </c>
       <c r="F38" t="n">
-        <v>0.0133779</v>
+        <v>0.0133466</v>
       </c>
       <c r="G38" t="n">
-        <v>0.004667900000000001</v>
+        <v>0.00461</v>
       </c>
     </row>
     <row r="39">
@@ -1431,19 +1431,19 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0.0005093000000000001</v>
+        <v>0.0005061</v>
       </c>
       <c r="D39" t="n">
-        <v>0.0019482</v>
+        <v>0.0021872</v>
       </c>
       <c r="E39" t="n">
-        <v>0.0090095</v>
+        <v>0.0127883</v>
       </c>
       <c r="F39" t="n">
-        <v>0.05484220000000001</v>
+        <v>0.08434139999999998</v>
       </c>
       <c r="G39" t="n">
-        <v>0.0165773</v>
+        <v>0.02495575</v>
       </c>
     </row>
     <row r="40">
@@ -1456,19 +1456,19 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0.0005922</v>
+        <v>0.0005546</v>
       </c>
       <c r="D40" t="n">
-        <v>0.0023443</v>
+        <v>0.0027382</v>
       </c>
       <c r="E40" t="n">
-        <v>0.0129631</v>
+        <v>0.0163032</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0861218</v>
+        <v>0.1224412</v>
       </c>
       <c r="G40" t="n">
-        <v>0.02550535</v>
+        <v>0.0355093</v>
       </c>
     </row>
     <row r="41">
@@ -1481,19 +1481,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0.0006981</v>
+        <v>0.000541</v>
       </c>
       <c r="D41" t="n">
-        <v>0.002830099999999999</v>
+        <v>0.002822</v>
       </c>
       <c r="E41" t="n">
-        <v>0.0139667</v>
+        <v>0.0177692</v>
       </c>
       <c r="F41" t="n">
-        <v>0.085648</v>
+        <v>0.1267977</v>
       </c>
       <c r="G41" t="n">
-        <v>0.025785725</v>
+        <v>0.036982475</v>
       </c>
     </row>
     <row r="42">
@@ -1506,19 +1506,19 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.000403</v>
+        <v>0.0004295</v>
       </c>
       <c r="D42" t="n">
-        <v>0.001654</v>
+        <v>0.0016831</v>
       </c>
       <c r="E42" t="n">
-        <v>0.0066898</v>
+        <v>0.006527599999999999</v>
       </c>
       <c r="F42" t="n">
-        <v>0.0271707</v>
+        <v>0.0270318</v>
       </c>
       <c r="G42" t="n">
-        <v>0.008979375</v>
+        <v>0.008918000000000001</v>
       </c>
     </row>
     <row r="43">
@@ -1531,19 +1531,19 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0.0006057</v>
+        <v>0.0005872000000000001</v>
       </c>
       <c r="D43" t="n">
-        <v>0.0028399</v>
+        <v>0.0030673</v>
       </c>
       <c r="E43" t="n">
-        <v>0.0179021</v>
+        <v>0.0204914</v>
       </c>
       <c r="F43" t="n">
-        <v>0.1528052</v>
+        <v>0.1945755</v>
       </c>
       <c r="G43" t="n">
-        <v>0.04353822500000001</v>
+        <v>0.05468035</v>
       </c>
     </row>
     <row r="44">
@@ -1556,19 +1556,19 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0.0003966</v>
+        <v>0.0003135999999999999</v>
       </c>
       <c r="D44" t="n">
-        <v>0.0011272</v>
+        <v>0.0009923</v>
       </c>
       <c r="E44" t="n">
-        <v>0.0032949</v>
+        <v>0.0027802</v>
       </c>
       <c r="F44" t="n">
-        <v>0.0106684</v>
+        <v>0.008577599999999999</v>
       </c>
       <c r="G44" t="n">
-        <v>0.003871775</v>
+        <v>0.003165925</v>
       </c>
     </row>
     <row r="45">
@@ -1581,19 +1581,19 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0.0004068</v>
+        <v>0.000273</v>
       </c>
       <c r="D45" t="n">
-        <v>0.0014149</v>
+        <v>0.0008062</v>
       </c>
       <c r="E45" t="n">
-        <v>0.0033747</v>
+        <v>0.002537</v>
       </c>
       <c r="F45" t="n">
-        <v>0.0117605</v>
+        <v>0.0092368</v>
       </c>
       <c r="G45" t="n">
-        <v>0.004239224999999999</v>
+        <v>0.00321325</v>
       </c>
     </row>
     <row r="46">
@@ -1606,19 +1606,19 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.0003226</v>
+        <v>0.0003198</v>
       </c>
       <c r="D46" t="n">
-        <v>0.0010937</v>
+        <v>0.0009858</v>
       </c>
       <c r="E46" t="n">
-        <v>0.0030327</v>
+        <v>0.0030054</v>
       </c>
       <c r="F46" t="n">
-        <v>0.0113453</v>
+        <v>0.0110127</v>
       </c>
       <c r="G46" t="n">
-        <v>0.003948574999999999</v>
+        <v>0.003830925</v>
       </c>
     </row>
     <row r="47">
@@ -1631,19 +1631,19 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0.0003851</v>
+        <v>0.0003623</v>
       </c>
       <c r="D47" t="n">
-        <v>0.0010217</v>
+        <v>0.001048</v>
       </c>
       <c r="E47" t="n">
-        <v>0.0027238</v>
+        <v>0.0032298</v>
       </c>
       <c r="F47" t="n">
-        <v>0.0114242</v>
+        <v>0.0111007</v>
       </c>
       <c r="G47" t="n">
-        <v>0.0038887</v>
+        <v>0.003935200000000001</v>
       </c>
     </row>
     <row r="48">
@@ -1656,19 +1656,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0.0007373</v>
+        <v>0.0005869</v>
       </c>
       <c r="D48" t="n">
-        <v>0.0029201</v>
+        <v>0.0029482</v>
       </c>
       <c r="E48" t="n">
-        <v>0.0142106</v>
+        <v>0.0179641</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0864718</v>
+        <v>0.126536</v>
       </c>
       <c r="G48" t="n">
-        <v>0.02608495</v>
+        <v>0.03700879999999999</v>
       </c>
     </row>
     <row r="49">
@@ -1681,19 +1681,19 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0.0004337</v>
+        <v>0.000325</v>
       </c>
       <c r="D49" t="n">
-        <v>0.001344</v>
+        <v>0.0008420000000000001</v>
       </c>
       <c r="E49" t="n">
-        <v>0.003318</v>
+        <v>0.0026129</v>
       </c>
       <c r="F49" t="n">
-        <v>0.0118754</v>
+        <v>0.009177299999999999</v>
       </c>
       <c r="G49" t="n">
-        <v>0.004242775</v>
+        <v>0.0032393</v>
       </c>
     </row>
   </sheetData>
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D4" t="n">
         <v>44</v>
@@ -1819,7 +1819,7 @@
         <v>176</v>
       </c>
       <c r="G4" t="n">
-        <v>82.5</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5">
@@ -1932,19 +1932,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D9" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E9" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="F9" t="n">
-        <v>176</v>
+        <v>194</v>
       </c>
       <c r="G9" t="n">
-        <v>82.5</v>
+        <v>90.5</v>
       </c>
     </row>
     <row r="10">
@@ -2032,7 +2032,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D13" t="n">
         <v>8</v>
@@ -2044,7 +2044,7 @@
         <v>9</v>
       </c>
       <c r="G13" t="n">
-        <v>8.5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
@@ -2182,19 +2182,19 @@
         </is>
       </c>
       <c r="C19" t="n">
+        <v>18</v>
+      </c>
+      <c r="D19" t="n">
         <v>19</v>
       </c>
-      <c r="D19" t="n">
-        <v>20</v>
-      </c>
       <c r="E19" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F19" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G19" t="n">
-        <v>20</v>
+        <v>18.75</v>
       </c>
     </row>
     <row r="20">
@@ -2282,19 +2282,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D23" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F23" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G23" t="n">
-        <v>8.5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24">
@@ -2307,19 +2307,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D24" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E24" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="F24" t="n">
-        <v>176</v>
+        <v>192</v>
       </c>
       <c r="G24" t="n">
-        <v>82.5</v>
+        <v>90</v>
       </c>
     </row>
     <row r="25">
@@ -2463,13 +2463,13 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F30" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G30" t="n">
-        <v>9.5</v>
+        <v>10.25</v>
       </c>
     </row>
     <row r="31">
@@ -2485,16 +2485,16 @@
         <v>22</v>
       </c>
       <c r="D31" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E31" t="n">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="F31" t="n">
-        <v>176</v>
+        <v>194</v>
       </c>
       <c r="G31" t="n">
-        <v>82.5</v>
+        <v>90</v>
       </c>
     </row>
     <row r="32">
@@ -2532,7 +2532,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D33" t="n">
         <v>20</v>
@@ -2541,7 +2541,7 @@
         <v>20</v>
       </c>
       <c r="F33" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G33" t="n">
         <v>19.25</v>
@@ -2607,19 +2607,19 @@
         </is>
       </c>
       <c r="C36" t="n">
+        <v>8</v>
+      </c>
+      <c r="D36" t="n">
         <v>10</v>
       </c>
-      <c r="D36" t="n">
-        <v>11</v>
-      </c>
       <c r="E36" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F36" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G36" t="n">
-        <v>11.75</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="37">
@@ -2682,19 +2682,19 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D39" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E39" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F39" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G39" t="n">
-        <v>8.5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="40">
@@ -2707,19 +2707,19 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D40" t="n">
         <v>10</v>
       </c>
       <c r="E40" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F40" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G40" t="n">
-        <v>10</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="41">
@@ -2732,19 +2732,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D41" t="n">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E41" t="n">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F41" t="n">
-        <v>176</v>
+        <v>198</v>
       </c>
       <c r="G41" t="n">
-        <v>82.5</v>
+        <v>92</v>
       </c>
     </row>
     <row r="42">
@@ -2785,16 +2785,16 @@
         <v>8</v>
       </c>
       <c r="D43" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F43" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G43" t="n">
-        <v>8</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="44">
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D44" t="n">
         <v>10</v>
@@ -2819,7 +2819,7 @@
         <v>11</v>
       </c>
       <c r="G44" t="n">
-        <v>10.25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45">
@@ -2832,7 +2832,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D45" t="n">
         <v>20</v>
@@ -2844,7 +2844,7 @@
         <v>20</v>
       </c>
       <c r="G45" t="n">
-        <v>19.25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="46">
@@ -2907,19 +2907,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D48" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E48" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F48" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G48" t="n">
-        <v>8</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="49">
@@ -2941,10 +2941,10 @@
         <v>10</v>
       </c>
       <c r="F49" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G49" t="n">
-        <v>10</v>
+        <v>9.75</v>
       </c>
     </row>
   </sheetData>
@@ -3058,19 +3058,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>25.55634918610405</v>
+        <v>28.38477631085023</v>
       </c>
       <c r="D4" t="n">
         <v>52.52691193458119</v>
       </c>
       <c r="E4" t="n">
-        <v>106.4680374315355</v>
+        <v>107.2964645562817</v>
       </c>
       <c r="F4" t="n">
         <v>214.350288425444</v>
       </c>
       <c r="G4" t="n">
-        <v>99.72539674441619</v>
+        <v>100.6396103067893</v>
       </c>
     </row>
     <row r="5">
@@ -3183,19 +3183,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>25.55634918610405</v>
+        <v>27.55634918610405</v>
       </c>
       <c r="D9" t="n">
-        <v>52.52691193458119</v>
+        <v>56.52691193458119</v>
       </c>
       <c r="E9" t="n">
-        <v>107.2964645562817</v>
+        <v>117.7817459305202</v>
       </c>
       <c r="F9" t="n">
-        <v>215.1787155501902</v>
+        <v>235.6639969244288</v>
       </c>
       <c r="G9" t="n">
-        <v>100.1396103067893</v>
+        <v>109.3822509939086</v>
       </c>
     </row>
     <row r="10">
@@ -3283,19 +3283,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>24.41488446708389</v>
+        <v>26.22000231742804</v>
       </c>
       <c r="D13" t="n">
         <v>49.56011556674471</v>
       </c>
       <c r="E13" t="n">
-        <v>101.1164142094206</v>
+        <v>100.6044505332257</v>
       </c>
       <c r="F13" t="n">
-        <v>203.2348880049742</v>
+        <v>202.7891131507078</v>
       </c>
       <c r="G13" t="n">
-        <v>94.58157556205583</v>
+        <v>94.79342039202658</v>
       </c>
     </row>
     <row r="14">
@@ -3339,13 +3339,13 @@
         <v>54.87005768508881</v>
       </c>
       <c r="E15" t="n">
-        <v>108.6690475583121</v>
+        <v>110.3259018078045</v>
       </c>
       <c r="F15" t="n">
-        <v>217.9238815542512</v>
+        <v>221.2375900532359</v>
       </c>
       <c r="G15" t="n">
-        <v>102.254833995939</v>
+        <v>103.4974746830583</v>
       </c>
     </row>
     <row r="16">
@@ -3433,19 +3433,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>27.55634918610405</v>
+        <v>25.55634918610405</v>
       </c>
       <c r="D19" t="n">
-        <v>54.04163056034262</v>
+        <v>51.69848480983499</v>
       </c>
       <c r="E19" t="n">
-        <v>108.6690475583121</v>
+        <v>103.9827560572969</v>
       </c>
       <c r="F19" t="n">
-        <v>223.4386001800126</v>
+        <v>208.5512985522207</v>
       </c>
       <c r="G19" t="n">
-        <v>103.4264068711929</v>
+        <v>97.44722215136414</v>
       </c>
     </row>
     <row r="20">
@@ -3533,19 +3533,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>24.41488446708389</v>
+        <v>26.4554706112443</v>
       </c>
       <c r="D23" t="n">
-        <v>49.60484583115361</v>
+        <v>52.67561329982938</v>
       </c>
       <c r="E23" t="n">
-        <v>101.1765739559945</v>
+        <v>108.790821278302</v>
       </c>
       <c r="F23" t="n">
-        <v>203.3015774098458</v>
+        <v>218.0487797413124</v>
       </c>
       <c r="G23" t="n">
-        <v>94.62447041601945</v>
+        <v>101.492671232672</v>
       </c>
     </row>
     <row r="24">
@@ -3558,19 +3558,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>25.55634918610405</v>
+        <v>27.55634918610405</v>
       </c>
       <c r="D24" t="n">
-        <v>52.52691193458119</v>
+        <v>56.52691193458119</v>
       </c>
       <c r="E24" t="n">
-        <v>106.4680374315355</v>
+        <v>116.953318805774</v>
       </c>
       <c r="F24" t="n">
-        <v>214.350288425444</v>
+        <v>232.8355697996826</v>
       </c>
       <c r="G24" t="n">
-        <v>99.72539674441619</v>
+        <v>108.4680374315355</v>
       </c>
     </row>
     <row r="25">
@@ -3583,7 +3583,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>27.55634918610405</v>
+        <v>26.72792206135786</v>
       </c>
       <c r="D25" t="n">
         <v>54.04163056034262</v>
@@ -3592,10 +3592,10 @@
         <v>109.4974746830583</v>
       </c>
       <c r="F25" t="n">
-        <v>218.7523086789974</v>
+        <v>222.0660171779821</v>
       </c>
       <c r="G25" t="n">
-        <v>102.4619407771256</v>
+        <v>103.0832611206852</v>
       </c>
     </row>
     <row r="26">
@@ -3692,10 +3692,10 @@
         <v>100.6044505332257</v>
       </c>
       <c r="F29" t="n">
-        <v>203.2348880049742</v>
+        <v>202.714772088272</v>
       </c>
       <c r="G29" t="n">
-        <v>94.45358464300712</v>
+        <v>94.32355566383158</v>
       </c>
     </row>
     <row r="30">
@@ -3714,13 +3714,13 @@
         <v>51.44598283082938</v>
       </c>
       <c r="E30" t="n">
-        <v>103.0023916359005</v>
+        <v>103.0999610655744</v>
       </c>
       <c r="F30" t="n">
-        <v>206.425148898921</v>
+        <v>207.3338489463796</v>
       </c>
       <c r="G30" t="n">
-        <v>96.6764618508823</v>
+        <v>96.92802922016543</v>
       </c>
     </row>
     <row r="31">
@@ -3736,16 +3736,16 @@
         <v>25.55634918610405</v>
       </c>
       <c r="D31" t="n">
-        <v>51.69848480983499</v>
+        <v>57.35533905932739</v>
       </c>
       <c r="E31" t="n">
-        <v>103.9827560572969</v>
+        <v>114.4680374315355</v>
       </c>
       <c r="F31" t="n">
-        <v>208.5512985522207</v>
+        <v>229.8650070512055</v>
       </c>
       <c r="G31" t="n">
-        <v>97.44722215136416</v>
+        <v>106.8111831820431</v>
       </c>
     </row>
     <row r="32">
@@ -3783,7 +3783,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>27.55634918610405</v>
+        <v>26.72792206135786</v>
       </c>
       <c r="D33" t="n">
         <v>54.04163056034262</v>
@@ -3792,10 +3792,10 @@
         <v>108.6690475583121</v>
       </c>
       <c r="F33" t="n">
-        <v>217.9238815542512</v>
+        <v>270.0243866176395</v>
       </c>
       <c r="G33" t="n">
-        <v>102.0477272147525</v>
+        <v>114.865746699413</v>
       </c>
     </row>
     <row r="34">
@@ -3858,19 +3858,19 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>26.59251907515131</v>
+        <v>24.62280887594792</v>
       </c>
       <c r="D36" t="n">
-        <v>52.62700551746683</v>
+        <v>50.84539750584248</v>
       </c>
       <c r="E36" t="n">
-        <v>105.9675221282317</v>
+        <v>101.6414365392452</v>
       </c>
       <c r="F36" t="n">
-        <v>222.6622168960765</v>
+        <v>204.0006534257569</v>
       </c>
       <c r="G36" t="n">
-        <v>101.9623159042316</v>
+        <v>95.27757408669811</v>
       </c>
     </row>
     <row r="37">
@@ -3933,19 +3933,19 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>24.41488446708389</v>
+        <v>26.4554706112443</v>
       </c>
       <c r="D39" t="n">
-        <v>49.56011556674471</v>
+        <v>52.67561329982938</v>
       </c>
       <c r="E39" t="n">
-        <v>100.6198800153907</v>
+        <v>108.790821278302</v>
       </c>
       <c r="F39" t="n">
-        <v>203.2568471454369</v>
+        <v>217.9744386788767</v>
       </c>
       <c r="G39" t="n">
-        <v>94.46293179866406</v>
+        <v>101.4740859670631</v>
       </c>
     </row>
     <row r="40">
@@ -3958,19 +3958,19 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>25.71936168599622</v>
+        <v>25.94223753527842</v>
       </c>
       <c r="D40" t="n">
-        <v>51.44598283082938</v>
+        <v>51.85071541632139</v>
       </c>
       <c r="E40" t="n">
-        <v>103.0999610655744</v>
+        <v>103.5721897488897</v>
       </c>
       <c r="F40" t="n">
-        <v>206.5701584477096</v>
+        <v>208.3389878701951</v>
       </c>
       <c r="G40" t="n">
-        <v>96.7088660075274</v>
+        <v>97.42603264267115</v>
       </c>
     </row>
     <row r="41">
@@ -3983,19 +3983,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>25.55634918610405</v>
+        <v>26.72792206135786</v>
       </c>
       <c r="D41" t="n">
-        <v>52.52691193458119</v>
+        <v>54.87005768508881</v>
       </c>
       <c r="E41" t="n">
-        <v>104.8111831820431</v>
+        <v>116.4680374315355</v>
       </c>
       <c r="F41" t="n">
-        <v>209.3797256769669</v>
+        <v>234.6934341759516</v>
       </c>
       <c r="G41" t="n">
-        <v>98.0685424949238</v>
+        <v>108.1898628384834</v>
       </c>
     </row>
     <row r="42">
@@ -4036,16 +4036,16 @@
         <v>24.41488446708389</v>
       </c>
       <c r="D43" t="n">
-        <v>49.03946295574199</v>
+        <v>53.5266090104926</v>
       </c>
       <c r="E43" t="n">
-        <v>98.78888910980251</v>
+        <v>106.9151001083049</v>
       </c>
       <c r="F43" t="n">
-        <v>198.4048488856638</v>
+        <v>214.3653506435532</v>
       </c>
       <c r="G43" t="n">
-        <v>92.66202135457306</v>
+        <v>99.80548605735865</v>
       </c>
     </row>
     <row r="44">
@@ -4058,19 +4058,19 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>26.59251907515131</v>
+        <v>25.94223753527842</v>
       </c>
       <c r="D44" t="n">
-        <v>52.12313371305741</v>
+        <v>52.1590137533636</v>
       </c>
       <c r="E44" t="n">
-        <v>104.9597785194129</v>
+        <v>104.3626331882609</v>
       </c>
       <c r="F44" t="n">
-        <v>210.8970608595957</v>
+        <v>216.807066810373</v>
       </c>
       <c r="G44" t="n">
-        <v>98.6431230418043</v>
+        <v>99.81773782181897</v>
       </c>
     </row>
     <row r="45">
@@ -4158,19 +4158,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>24.41488446708389</v>
+        <v>25.94223753527842</v>
       </c>
       <c r="D48" t="n">
-        <v>49.21635711250729</v>
+        <v>52.2265241682892</v>
       </c>
       <c r="E48" t="n">
-        <v>98.78888910980251</v>
+        <v>107.5808111303428</v>
       </c>
       <c r="F48" t="n">
-        <v>198.4048488856638</v>
+        <v>218.0501723215458</v>
       </c>
       <c r="G48" t="n">
-        <v>92.70624489376438</v>
+        <v>100.9499362888641</v>
       </c>
     </row>
     <row r="49">
@@ -4183,19 +4183,19 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>25.71936168599622</v>
+        <v>25.94223753527842</v>
       </c>
       <c r="D49" t="n">
-        <v>52.12313371305741</v>
+        <v>52.1590137533636</v>
       </c>
       <c r="E49" t="n">
-        <v>104.9597785194129</v>
+        <v>104.3626331882609</v>
       </c>
       <c r="F49" t="n">
-        <v>210.8970608595957</v>
+        <v>209.4868100138525</v>
       </c>
       <c r="G49" t="n">
-        <v>98.42483369451554</v>
+        <v>97.98767362268885</v>
       </c>
     </row>
   </sheetData>
@@ -4309,19 +4309,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D4" t="n">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="E4" t="n">
-        <v>276</v>
+        <v>331</v>
       </c>
       <c r="F4" t="n">
-        <v>606</v>
+        <v>836</v>
       </c>
       <c r="G4" t="n">
-        <v>252.75</v>
+        <v>327.75</v>
       </c>
     </row>
     <row r="5">
@@ -4434,19 +4434,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D9" t="n">
-        <v>107</v>
+        <v>140</v>
       </c>
       <c r="E9" t="n">
-        <v>287</v>
+        <v>396</v>
       </c>
       <c r="F9" t="n">
-        <v>616</v>
+        <v>1009</v>
       </c>
       <c r="G9" t="n">
-        <v>262</v>
+        <v>396.75</v>
       </c>
     </row>
     <row r="10">
@@ -4534,19 +4534,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D13" t="n">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="E13" t="n">
-        <v>276</v>
+        <v>331</v>
       </c>
       <c r="F13" t="n">
-        <v>606</v>
+        <v>836</v>
       </c>
       <c r="G13" t="n">
-        <v>252.75</v>
+        <v>327.75</v>
       </c>
     </row>
     <row r="14">
@@ -4562,16 +4562,16 @@
         <v>33</v>
       </c>
       <c r="D14" t="n">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="E14" t="n">
-        <v>256</v>
+        <v>365</v>
       </c>
       <c r="F14" t="n">
-        <v>628</v>
+        <v>833</v>
       </c>
       <c r="G14" t="n">
-        <v>253</v>
+        <v>333.25</v>
       </c>
     </row>
     <row r="15">
@@ -4587,16 +4587,16 @@
         <v>29</v>
       </c>
       <c r="D15" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E15" t="n">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="F15" t="n">
-        <v>455</v>
+        <v>432</v>
       </c>
       <c r="G15" t="n">
-        <v>196.25</v>
+        <v>189.25</v>
       </c>
     </row>
     <row r="16">
@@ -4684,16 +4684,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D19" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E19" t="n">
         <v>13</v>
       </c>
       <c r="F19" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G19" t="n">
         <v>12.75</v>
@@ -4784,19 +4784,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D23" t="n">
-        <v>107</v>
+        <v>140</v>
       </c>
       <c r="E23" t="n">
-        <v>287</v>
+        <v>396</v>
       </c>
       <c r="F23" t="n">
-        <v>616</v>
+        <v>1009</v>
       </c>
       <c r="G23" t="n">
-        <v>262</v>
+        <v>396.75</v>
       </c>
     </row>
     <row r="24">
@@ -4809,19 +4809,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D24" t="n">
-        <v>92</v>
+        <v>145</v>
       </c>
       <c r="E24" t="n">
-        <v>249</v>
+        <v>427</v>
       </c>
       <c r="F24" t="n">
-        <v>508</v>
+        <v>1001</v>
       </c>
       <c r="G24" t="n">
-        <v>220.75</v>
+        <v>403.75</v>
       </c>
     </row>
     <row r="25">
@@ -4834,19 +4834,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D25" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="E25" t="n">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="F25" t="n">
-        <v>475</v>
+        <v>494</v>
       </c>
       <c r="G25" t="n">
-        <v>207.25</v>
+        <v>213.25</v>
       </c>
     </row>
     <row r="26">
@@ -4937,16 +4937,16 @@
         <v>33</v>
       </c>
       <c r="D29" t="n">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="E29" t="n">
-        <v>256</v>
+        <v>365</v>
       </c>
       <c r="F29" t="n">
-        <v>628</v>
+        <v>833</v>
       </c>
       <c r="G29" t="n">
-        <v>253</v>
+        <v>333.25</v>
       </c>
     </row>
     <row r="30">
@@ -4962,16 +4962,16 @@
         <v>29</v>
       </c>
       <c r="D30" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E30" t="n">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="F30" t="n">
-        <v>455</v>
+        <v>432</v>
       </c>
       <c r="G30" t="n">
-        <v>196.25</v>
+        <v>189.25</v>
       </c>
     </row>
     <row r="31">
@@ -4987,16 +4987,16 @@
         <v>28</v>
       </c>
       <c r="D31" t="n">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="E31" t="n">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F31" t="n">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="G31" t="n">
-        <v>221.5</v>
+        <v>226.75</v>
       </c>
     </row>
     <row r="32">
@@ -5034,19 +5034,19 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D33" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E33" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F33" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G33" t="n">
-        <v>15.75</v>
+        <v>16.75</v>
       </c>
     </row>
     <row r="34">
@@ -5109,16 +5109,16 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D36" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E36" t="n">
         <v>13</v>
       </c>
       <c r="F36" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G36" t="n">
         <v>12.75</v>
@@ -5137,16 +5137,16 @@
         <v>12</v>
       </c>
       <c r="D37" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E37" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F37" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G37" t="n">
-        <v>12</v>
+        <v>13.75</v>
       </c>
     </row>
     <row r="38">
@@ -5184,19 +5184,19 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="D39" t="n">
-        <v>92</v>
+        <v>145</v>
       </c>
       <c r="E39" t="n">
-        <v>249</v>
+        <v>427</v>
       </c>
       <c r="F39" t="n">
-        <v>508</v>
+        <v>1001</v>
       </c>
       <c r="G39" t="n">
-        <v>220.75</v>
+        <v>403.75</v>
       </c>
     </row>
     <row r="40">
@@ -5209,19 +5209,19 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D40" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="E40" t="n">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="F40" t="n">
-        <v>475</v>
+        <v>494</v>
       </c>
       <c r="G40" t="n">
-        <v>207.25</v>
+        <v>213.25</v>
       </c>
     </row>
     <row r="41">
@@ -5234,19 +5234,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="D41" t="n">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="E41" t="n">
-        <v>279</v>
+        <v>318</v>
       </c>
       <c r="F41" t="n">
-        <v>605</v>
+        <v>675</v>
       </c>
       <c r="G41" t="n">
-        <v>259.5</v>
+        <v>282.5</v>
       </c>
     </row>
     <row r="42">
@@ -5287,16 +5287,16 @@
         <v>28</v>
       </c>
       <c r="D43" t="n">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="E43" t="n">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F43" t="n">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="G43" t="n">
-        <v>221.5</v>
+        <v>226.75</v>
       </c>
     </row>
     <row r="44">
@@ -5309,19 +5309,19 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D44" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E44" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F44" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G44" t="n">
-        <v>15.75</v>
+        <v>16.75</v>
       </c>
     </row>
     <row r="45">
@@ -5337,13 +5337,13 @@
         <v>13</v>
       </c>
       <c r="D45" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E45" t="n">
         <v>18</v>
       </c>
       <c r="F45" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G45" t="n">
         <v>17</v>
@@ -5387,16 +5387,16 @@
         <v>12</v>
       </c>
       <c r="D47" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E47" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F47" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G47" t="n">
-        <v>12</v>
+        <v>13.75</v>
       </c>
     </row>
     <row r="48">
@@ -5409,19 +5409,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="D48" t="n">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="E48" t="n">
-        <v>279</v>
+        <v>318</v>
       </c>
       <c r="F48" t="n">
-        <v>605</v>
+        <v>675</v>
       </c>
       <c r="G48" t="n">
-        <v>259.5</v>
+        <v>282.5</v>
       </c>
     </row>
     <row r="49">
@@ -5437,13 +5437,13 @@
         <v>13</v>
       </c>
       <c r="D49" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E49" t="n">
         <v>18</v>
       </c>
       <c r="F49" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G49" t="n">
         <v>17</v>
@@ -5560,19 +5560,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D4" t="n">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E4" t="n">
-        <v>365</v>
+        <v>395</v>
       </c>
       <c r="F4" t="n">
-        <v>2113</v>
+        <v>1847</v>
       </c>
       <c r="G4" t="n">
-        <v>646.75</v>
+        <v>588</v>
       </c>
     </row>
     <row r="5">
@@ -5685,19 +5685,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D9" t="n">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="E9" t="n">
-        <v>463</v>
+        <v>494</v>
       </c>
       <c r="F9" t="n">
-        <v>1824</v>
+        <v>2034</v>
       </c>
       <c r="G9" t="n">
-        <v>613</v>
+        <v>668.75</v>
       </c>
     </row>
     <row r="10">
@@ -5785,19 +5785,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D13" t="n">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E13" t="n">
-        <v>365</v>
+        <v>395</v>
       </c>
       <c r="F13" t="n">
-        <v>2113</v>
+        <v>1847</v>
       </c>
       <c r="G13" t="n">
-        <v>646.75</v>
+        <v>588</v>
       </c>
     </row>
     <row r="14">
@@ -5810,19 +5810,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D14" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E14" t="n">
-        <v>353</v>
+        <v>439</v>
       </c>
       <c r="F14" t="n">
-        <v>2096</v>
+        <v>2007</v>
       </c>
       <c r="G14" t="n">
-        <v>639.75</v>
+        <v>636.75</v>
       </c>
     </row>
     <row r="15">
@@ -5835,19 +5835,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D15" t="n">
         <v>110</v>
       </c>
       <c r="E15" t="n">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="F15" t="n">
-        <v>2444</v>
+        <v>2368</v>
       </c>
       <c r="G15" t="n">
-        <v>767.75</v>
+        <v>748.75</v>
       </c>
     </row>
     <row r="16">
@@ -5938,16 +5938,16 @@
         <v>20</v>
       </c>
       <c r="D19" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E19" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F19" t="n">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G19" t="n">
-        <v>31.25</v>
+        <v>29.75</v>
       </c>
     </row>
     <row r="20">
@@ -6035,19 +6035,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D23" t="n">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="E23" t="n">
-        <v>463</v>
+        <v>494</v>
       </c>
       <c r="F23" t="n">
-        <v>1824</v>
+        <v>2034</v>
       </c>
       <c r="G23" t="n">
-        <v>613</v>
+        <v>668.75</v>
       </c>
     </row>
     <row r="24">
@@ -6060,19 +6060,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D24" t="n">
-        <v>128</v>
+        <v>107</v>
       </c>
       <c r="E24" t="n">
-        <v>478</v>
+        <v>498</v>
       </c>
       <c r="F24" t="n">
-        <v>1954</v>
+        <v>1977</v>
       </c>
       <c r="G24" t="n">
-        <v>650</v>
+        <v>654</v>
       </c>
     </row>
     <row r="25">
@@ -6085,19 +6085,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="D25" t="n">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="E25" t="n">
-        <v>605</v>
+        <v>586</v>
       </c>
       <c r="F25" t="n">
-        <v>2384</v>
+        <v>2504</v>
       </c>
       <c r="G25" t="n">
-        <v>800</v>
+        <v>819.75</v>
       </c>
     </row>
     <row r="26">
@@ -6185,19 +6185,19 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D29" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E29" t="n">
-        <v>353</v>
+        <v>439</v>
       </c>
       <c r="F29" t="n">
-        <v>2096</v>
+        <v>2007</v>
       </c>
       <c r="G29" t="n">
-        <v>639.75</v>
+        <v>636.75</v>
       </c>
     </row>
     <row r="30">
@@ -6210,19 +6210,19 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D30" t="n">
         <v>110</v>
       </c>
       <c r="E30" t="n">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="F30" t="n">
-        <v>2444</v>
+        <v>2368</v>
       </c>
       <c r="G30" t="n">
-        <v>767.75</v>
+        <v>748.75</v>
       </c>
     </row>
     <row r="31">
@@ -6235,19 +6235,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D31" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E31" t="n">
-        <v>454</v>
+        <v>478</v>
       </c>
       <c r="F31" t="n">
-        <v>2132</v>
+        <v>2594</v>
       </c>
       <c r="G31" t="n">
-        <v>683.25</v>
+        <v>804.5</v>
       </c>
     </row>
     <row r="32">
@@ -6285,19 +6285,19 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D33" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="E33" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="F33" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="G33" t="n">
-        <v>34.5</v>
+        <v>25.75</v>
       </c>
     </row>
     <row r="34">
@@ -6363,16 +6363,16 @@
         <v>20</v>
       </c>
       <c r="D36" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E36" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F36" t="n">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G36" t="n">
-        <v>31.25</v>
+        <v>29.75</v>
       </c>
     </row>
     <row r="37">
@@ -6385,19 +6385,19 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D37" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E37" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F37" t="n">
         <v>38</v>
       </c>
       <c r="G37" t="n">
-        <v>31</v>
+        <v>33.25</v>
       </c>
     </row>
     <row r="38">
@@ -6435,19 +6435,19 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D39" t="n">
-        <v>128</v>
+        <v>107</v>
       </c>
       <c r="E39" t="n">
-        <v>478</v>
+        <v>498</v>
       </c>
       <c r="F39" t="n">
-        <v>1954</v>
+        <v>1977</v>
       </c>
       <c r="G39" t="n">
-        <v>650</v>
+        <v>654</v>
       </c>
     </row>
     <row r="40">
@@ -6460,19 +6460,19 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="D40" t="n">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="E40" t="n">
-        <v>605</v>
+        <v>586</v>
       </c>
       <c r="F40" t="n">
-        <v>2384</v>
+        <v>2504</v>
       </c>
       <c r="G40" t="n">
-        <v>800</v>
+        <v>819.75</v>
       </c>
     </row>
     <row r="41">
@@ -6485,19 +6485,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="D41" t="n">
-        <v>177</v>
+        <v>147</v>
       </c>
       <c r="E41" t="n">
-        <v>657</v>
+        <v>616</v>
       </c>
       <c r="F41" t="n">
-        <v>2515</v>
+        <v>2588</v>
       </c>
       <c r="G41" t="n">
-        <v>851.75</v>
+        <v>848</v>
       </c>
     </row>
     <row r="42">
@@ -6535,19 +6535,19 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D43" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E43" t="n">
-        <v>454</v>
+        <v>478</v>
       </c>
       <c r="F43" t="n">
-        <v>2132</v>
+        <v>2594</v>
       </c>
       <c r="G43" t="n">
-        <v>683.25</v>
+        <v>804.5</v>
       </c>
     </row>
     <row r="44">
@@ -6560,19 +6560,19 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D44" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="E44" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="F44" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="G44" t="n">
-        <v>34.5</v>
+        <v>25.75</v>
       </c>
     </row>
     <row r="45">
@@ -6585,19 +6585,19 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D45" t="n">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E45" t="n">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="F45" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="G45" t="n">
-        <v>35.75</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="46">
@@ -6635,19 +6635,19 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D47" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E47" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F47" t="n">
         <v>38</v>
       </c>
       <c r="G47" t="n">
-        <v>31</v>
+        <v>33.25</v>
       </c>
     </row>
     <row r="48">
@@ -6660,19 +6660,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="D48" t="n">
-        <v>177</v>
+        <v>147</v>
       </c>
       <c r="E48" t="n">
-        <v>657</v>
+        <v>616</v>
       </c>
       <c r="F48" t="n">
-        <v>2515</v>
+        <v>2588</v>
       </c>
       <c r="G48" t="n">
-        <v>851.75</v>
+        <v>848</v>
       </c>
     </row>
     <row r="49">
@@ -6685,19 +6685,19 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D49" t="n">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E49" t="n">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="F49" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="G49" t="n">
-        <v>35.75</v>
+        <v>25.5</v>
       </c>
     </row>
   </sheetData>
@@ -6814,10 +6814,10 @@
         <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F4" t="n">
         <v>24</v>
@@ -6939,16 +6939,16 @@
         <v>11</v>
       </c>
       <c r="D9" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E9" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F9" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G9" t="n">
-        <v>14.25</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="10">
@@ -7036,7 +7036,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D13" t="n">
         <v>6</v>
@@ -7048,7 +7048,7 @@
         <v>7</v>
       </c>
       <c r="G13" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -7061,19 +7061,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D14" t="n">
         <v>12</v>
       </c>
       <c r="E14" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F14" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G14" t="n">
-        <v>13.75</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="15">
@@ -7086,19 +7086,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D15" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E15" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F15" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="G15" t="n">
-        <v>18.75</v>
+        <v>21.75</v>
       </c>
     </row>
     <row r="16">
@@ -7186,19 +7186,19 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D19" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E19" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F19" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G19" t="n">
-        <v>13.5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20">
@@ -7286,19 +7286,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D23" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E23" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F23" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G23" t="n">
-        <v>6.5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24">
@@ -7314,16 +7314,16 @@
         <v>11</v>
       </c>
       <c r="D24" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E24" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F24" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G24" t="n">
-        <v>12.25</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="25">
@@ -7336,19 +7336,19 @@
         </is>
       </c>
       <c r="C25" t="n">
+        <v>10</v>
+      </c>
+      <c r="D25" t="n">
+        <v>12</v>
+      </c>
+      <c r="E25" t="n">
         <v>16</v>
       </c>
-      <c r="D25" t="n">
-        <v>16</v>
-      </c>
-      <c r="E25" t="n">
-        <v>24</v>
-      </c>
       <c r="F25" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G25" t="n">
-        <v>21</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="26">
@@ -7467,13 +7467,13 @@
         <v>8</v>
       </c>
       <c r="E30" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F30" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G30" t="n">
-        <v>7.5</v>
+        <v>8.25</v>
       </c>
     </row>
     <row r="31">
@@ -7486,19 +7486,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D31" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E31" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F31" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="G31" t="n">
-        <v>11.75</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="32">
@@ -7536,19 +7536,19 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D33" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E33" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F33" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G33" t="n">
-        <v>13.75</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="34">
@@ -7611,19 +7611,19 @@
         </is>
       </c>
       <c r="C36" t="n">
+        <v>6</v>
+      </c>
+      <c r="D36" t="n">
         <v>8</v>
       </c>
-      <c r="D36" t="n">
-        <v>9</v>
-      </c>
       <c r="E36" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F36" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G36" t="n">
-        <v>9.75</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="37">
@@ -7686,19 +7686,19 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D39" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E39" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F39" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G39" t="n">
-        <v>6.5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="40">
@@ -7717,13 +7717,13 @@
         <v>8</v>
       </c>
       <c r="E40" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F40" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G40" t="n">
-        <v>7.75</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="41">
@@ -7736,19 +7736,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D41" t="n">
         <v>13</v>
       </c>
       <c r="E41" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F41" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="G41" t="n">
-        <v>13.5</v>
+        <v>15.75</v>
       </c>
     </row>
     <row r="42">
@@ -7789,16 +7789,16 @@
         <v>6</v>
       </c>
       <c r="D43" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E43" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F43" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G43" t="n">
-        <v>6</v>
+        <v>8.25</v>
       </c>
     </row>
     <row r="44">
@@ -7811,7 +7811,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D44" t="n">
         <v>8</v>
@@ -7823,7 +7823,7 @@
         <v>9</v>
       </c>
       <c r="G44" t="n">
-        <v>8.25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="45">
@@ -7836,19 +7836,19 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D45" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E45" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F45" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G45" t="n">
-        <v>13.75</v>
+        <v>11.75</v>
       </c>
     </row>
     <row r="46">
@@ -7911,19 +7911,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D48" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E48" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F48" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G48" t="n">
-        <v>6</v>
+        <v>8.25</v>
       </c>
     </row>
     <row r="49">
@@ -7945,10 +7945,10 @@
         <v>8</v>
       </c>
       <c r="F49" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G49" t="n">
-        <v>8</v>
+        <v>7.75</v>
       </c>
     </row>
   </sheetData>
@@ -8037,16 +8037,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="C4" t="n">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="D4" t="n">
-        <v>641</v>
+        <v>726</v>
       </c>
       <c r="E4" t="n">
-        <v>2719</v>
+        <v>2683</v>
       </c>
     </row>
     <row r="5">
@@ -8132,16 +8132,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C9" t="n">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="D9" t="n">
-        <v>750</v>
+        <v>890</v>
       </c>
       <c r="E9" t="n">
-        <v>2440</v>
+        <v>3043</v>
       </c>
     </row>
     <row r="10">
@@ -8208,16 +8208,16 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="C13" t="n">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="D13" t="n">
-        <v>641</v>
+        <v>726</v>
       </c>
       <c r="E13" t="n">
-        <v>2719</v>
+        <v>2683</v>
       </c>
     </row>
     <row r="14">
@@ -8227,16 +8227,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C14" t="n">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D14" t="n">
-        <v>609</v>
+        <v>804</v>
       </c>
       <c r="E14" t="n">
-        <v>2724</v>
+        <v>2840</v>
       </c>
     </row>
     <row r="15">
@@ -8246,16 +8246,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C15" t="n">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D15" t="n">
-        <v>689</v>
+        <v>685</v>
       </c>
       <c r="E15" t="n">
-        <v>2899</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="16">
@@ -8322,16 +8322,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C19" t="n">
         <v>42</v>
       </c>
       <c r="D19" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E19" t="n">
-        <v>57</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20">
@@ -8398,16 +8398,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C23" t="n">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="D23" t="n">
-        <v>750</v>
+        <v>890</v>
       </c>
       <c r="E23" t="n">
-        <v>2440</v>
+        <v>3043</v>
       </c>
     </row>
     <row r="24">
@@ -8417,16 +8417,16 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C24" t="n">
-        <v>220</v>
+        <v>252</v>
       </c>
       <c r="D24" t="n">
-        <v>727</v>
+        <v>925</v>
       </c>
       <c r="E24" t="n">
-        <v>2462</v>
+        <v>2978</v>
       </c>
     </row>
     <row r="25">
@@ -8436,16 +8436,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="C25" t="n">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D25" t="n">
-        <v>835</v>
+        <v>809</v>
       </c>
       <c r="E25" t="n">
-        <v>2859</v>
+        <v>2998</v>
       </c>
     </row>
     <row r="26">
@@ -8512,16 +8512,16 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C29" t="n">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D29" t="n">
-        <v>609</v>
+        <v>804</v>
       </c>
       <c r="E29" t="n">
-        <v>2724</v>
+        <v>2840</v>
       </c>
     </row>
     <row r="30">
@@ -8531,16 +8531,16 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C30" t="n">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D30" t="n">
-        <v>689</v>
+        <v>685</v>
       </c>
       <c r="E30" t="n">
-        <v>2899</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="31">
@@ -8550,16 +8550,16 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C31" t="n">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="D31" t="n">
-        <v>688</v>
+        <v>713</v>
       </c>
       <c r="E31" t="n">
-        <v>2663</v>
+        <v>3131</v>
       </c>
     </row>
     <row r="32">
@@ -8588,16 +8588,16 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C33" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D33" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E33" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34">
@@ -8645,16 +8645,16 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C36" t="n">
         <v>42</v>
       </c>
       <c r="D36" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E36" t="n">
-        <v>57</v>
+        <v>50</v>
       </c>
     </row>
     <row r="37">
@@ -8664,16 +8664,16 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C37" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D37" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E37" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="38">
@@ -8702,16 +8702,16 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C39" t="n">
-        <v>220</v>
+        <v>252</v>
       </c>
       <c r="D39" t="n">
-        <v>727</v>
+        <v>925</v>
       </c>
       <c r="E39" t="n">
-        <v>2462</v>
+        <v>2978</v>
       </c>
     </row>
     <row r="40">
@@ -8721,16 +8721,16 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="C40" t="n">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D40" t="n">
-        <v>835</v>
+        <v>809</v>
       </c>
       <c r="E40" t="n">
-        <v>2859</v>
+        <v>2998</v>
       </c>
     </row>
     <row r="41">
@@ -8740,16 +8740,16 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="C41" t="n">
-        <v>295</v>
+        <v>256</v>
       </c>
       <c r="D41" t="n">
-        <v>936</v>
+        <v>934</v>
       </c>
       <c r="E41" t="n">
-        <v>3120</v>
+        <v>3263</v>
       </c>
     </row>
     <row r="42">
@@ -8778,16 +8778,16 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C43" t="n">
-        <v>201</v>
+        <v>218</v>
       </c>
       <c r="D43" t="n">
-        <v>688</v>
+        <v>713</v>
       </c>
       <c r="E43" t="n">
-        <v>2663</v>
+        <v>3131</v>
       </c>
     </row>
     <row r="44">
@@ -8797,16 +8797,16 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C44" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D44" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E44" t="n">
-        <v>53</v>
+        <v>41</v>
       </c>
     </row>
     <row r="45">
@@ -8816,16 +8816,16 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C45" t="n">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="D45" t="n">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="E45" t="n">
-        <v>57</v>
+        <v>46</v>
       </c>
     </row>
     <row r="46">
@@ -8854,16 +8854,16 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C47" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D47" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="E47" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="48">
@@ -8873,16 +8873,16 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="C48" t="n">
-        <v>295</v>
+        <v>256</v>
       </c>
       <c r="D48" t="n">
-        <v>936</v>
+        <v>934</v>
       </c>
       <c r="E48" t="n">
-        <v>3120</v>
+        <v>3263</v>
       </c>
     </row>
     <row r="49">
@@ -8892,16 +8892,16 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C49" t="n">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="D49" t="n">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="E49" t="n">
-        <v>57</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>